<commit_message>
Criação inicial do projeto
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75247B1C-706E-454F-871D-C3A702E35A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A62FC60-0AC5-40F5-AFCF-73DB8DC8243D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{59D4C9AA-0B45-4A22-B6BD-D08E6C242389}"/>
   </bookViews>
@@ -31,6 +31,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -83,19 +86,19 @@
     <t>Tasks</t>
   </si>
   <si>
-    <t>Baixar sql server</t>
-  </si>
-  <si>
     <t>Modelar banco de dados</t>
   </si>
   <si>
-    <t>Criar design telas</t>
-  </si>
-  <si>
-    <t>Criar github</t>
-  </si>
-  <si>
-    <t>Criar projeto MVC</t>
+    <t>Eu como usuário quero poder criar conta, excluir, editar informações da aplicação</t>
+  </si>
+  <si>
+    <t>Eu como usuário quero ver os produtos novos que chegaram na loja</t>
+  </si>
+  <si>
+    <t>Eu como usuário quero visualizar recomendações, com base nas minhas últimas compras</t>
+  </si>
+  <si>
+    <t>Criar algoritmo que análise compras de outros usuários do site e recomende produtos que esses outros usuários também compraram junto ou em outro momento</t>
   </si>
 </sst>
 </file>
@@ -119,12 +122,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -139,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -148,17 +157,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -494,7 +506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0855CDB-E763-4D95-8CC1-C9E4FEECBA91}">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.7109375" style="3" customWidth="1"/>
@@ -510,15 +522,15 @@
       </c>
     </row>
     <row r="2" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5"/>
-      <c r="B2" s="4" t="s">
+      <c r="A2" s="6"/>
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="6"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="4"/>
+      <c r="C2" s="4"/>
+    </row>
+    <row r="3" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="B3" s="5"/>
     </row>
     <row r="4" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
@@ -565,59 +577,65 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B14" s="3" t="s">
+    <row r="16" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="4" t="s">
+    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="7"/>
+      <c r="B17" s="5" t="s">
         <v>13</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="3" t="s">
-        <v>18</v>
+      <c r="B18" s="5"/>
+      <c r="C18" s="8" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="7"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="3" t="s">
-        <v>19</v>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="7"/>
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="7"/>
+      <c r="B21" s="5"/>
+    </row>
+    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B22" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B15:B19"/>
-    <mergeCell ref="A15:A19"/>
+    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="A17:A21"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
EM-3.1 - Criação da tela principal da aplicação
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A62FC60-0AC5-40F5-AFCF-73DB8DC8243D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D2DD09B-8EB2-49AC-BDD9-10F3773C784C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{59D4C9AA-0B45-4A22-B6BD-D08E6C242389}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>US</t>
   </si>
@@ -53,9 +53,6 @@
     <t>Eu como usuário quero visualizar o catálogo de produtos por tipo, marca,  ofertas</t>
   </si>
   <si>
-    <t>Eu como usuário quero poder filtrar os produtos</t>
-  </si>
-  <si>
     <t>Eu como usuário quero armazenar os produtos em um carrinho de compras e realizar a compra posteriormente de forma segura</t>
   </si>
   <si>
@@ -99,6 +96,120 @@
   </si>
   <si>
     <t>Criar algoritmo que análise compras de outros usuários do site e recomende produtos que esses outros usuários também compraram junto ou em outro momento</t>
+  </si>
+  <si>
+    <t>Definir as tarefas de cada uma das US</t>
+  </si>
+  <si>
+    <t>Criação de tela para cadastro dos produtos</t>
+  </si>
+  <si>
+    <t>Criação de rotina para cadastro de produto no banco de dados</t>
+  </si>
+  <si>
+    <t>Criar tela para importar excel</t>
+  </si>
+  <si>
+    <t>Criar rotina para importar informações do excel</t>
+  </si>
+  <si>
+    <t>Criar rotina para importar imagens das roupas, através de um zip, ou através de uma url cadastrada no excel (armazenar as imagens em um ftp e cadastrar no banco de dados somente a url)</t>
+  </si>
+  <si>
+    <t>Criar tela com filtro e grade de produtos</t>
+  </si>
+  <si>
+    <t>Criar filtro na tela principal</t>
+  </si>
+  <si>
+    <t>Criar na tela principal a visualização de um carrinho de compras</t>
+  </si>
+  <si>
+    <t>Criar rotina para armazenar os produtos selecionados em cache (REDIS)</t>
+  </si>
+  <si>
+    <t>Criar tela para finalização da compra</t>
+  </si>
+  <si>
+    <t>Criar rotina para pagamento, integração com meios de pagamentos</t>
+  </si>
+  <si>
+    <t>Criar rotina para alerta por email das ofertas, email disparado de forma automática ou manual pelo administrador</t>
+  </si>
+  <si>
+    <t>Criar tela para programar os alertas e disparar alertas manuais</t>
+  </si>
+  <si>
+    <t>Criar rotina para calcular o frete</t>
+  </si>
+  <si>
+    <t>Incluir na tela de finalização das compras o valor do frete</t>
+  </si>
+  <si>
+    <t>Criar tela para cadastro de promoções</t>
+  </si>
+  <si>
+    <t>Definir quais os tipos de promoções vão estar disponiveis para cadastro</t>
+  </si>
+  <si>
+    <t>Rotina de integração com o google</t>
+  </si>
+  <si>
+    <t>Na tela de edição dos produtos, ter como definir flag para destacar produto</t>
+  </si>
+  <si>
+    <t>Na tela principal ter disponivel sessão com os produtos novos</t>
+  </si>
+  <si>
+    <t>Criar tela para exibir ao usuário as compras realizadas e status</t>
+  </si>
+  <si>
+    <t>Criar rotina para envio de email sempre que houver atualização no status</t>
+  </si>
+  <si>
+    <t>Criar tela de login</t>
+  </si>
+  <si>
+    <t>Criar tela de cadastro</t>
+  </si>
+  <si>
+    <t>Criar tela de edição</t>
+  </si>
+  <si>
+    <t>Criar rotina de login</t>
+  </si>
+  <si>
+    <t>Criar rotina de cadastro</t>
+  </si>
+  <si>
+    <t>Criar rotina de edição</t>
+  </si>
+  <si>
+    <t>Criar tela principal</t>
+  </si>
+  <si>
+    <t>3.1</t>
+  </si>
+  <si>
+    <t>10.1</t>
+  </si>
+  <si>
+    <t>4.1</t>
+  </si>
+  <si>
+    <t>Definir melhor a forma como armazenar imagens para a aplicação</t>
+  </si>
+  <si>
+    <t>1.1</t>
+  </si>
+  <si>
+    <t>Criar lógica para retornar produtos para a tela principal</t>
+  </si>
+  <si>
+    <t>3.2</t>
+  </si>
+  <si>
+    <t>Criar tela para listar os produtos femininos</t>
   </si>
 </sst>
 </file>
@@ -148,30 +259,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -506,136 +621,375 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0855CDB-E763-4D95-8CC1-C9E4FEECBA91}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="42.7109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="37.28515625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="4"/>
+    <col min="2" max="2" width="42.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="37.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4"/>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="9"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="9">
+        <v>2</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="96.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="9"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="9"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="9">
+        <v>3</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="9"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="9"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="9"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="9"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="9">
+        <v>4</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="9"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="9"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="9"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="9">
+        <v>5</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="9"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9">
+        <v>6</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="9"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="9">
+        <v>7</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="9"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="4">
+        <v>8</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="4">
+        <v>9</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
+        <v>10</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A26" s="4">
+        <v>11</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="4">
+        <v>12</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="4">
+        <v>13</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="9">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6"/>
-      <c r="B2" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="4"/>
-    </row>
-    <row r="3" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="5"/>
-    </row>
-    <row r="4" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B4" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B5" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B6" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B8" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B9" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="B10" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B11" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="B12" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="B14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="3" t="s">
+      <c r="B29" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="9"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="9"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B15" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B16" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="8" t="s">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="9"/>
+      <c r="B32" s="8"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="9"/>
+      <c r="B33" s="8"/>
+    </row>
+    <row r="34" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="9">
         <v>15</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
-      <c r="B19" s="5"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="5"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="5"/>
-    </row>
-    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B22" s="3" t="s">
-        <v>16</v>
+      <c r="B34" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="9"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="9"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="9"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="9"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="9"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="A17:A21"/>
+  <mergeCells count="18">
+    <mergeCell ref="B34:B39"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A34:A39"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B29:B33"/>
+    <mergeCell ref="A29:A33"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B21:B22"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
EM-3.2 - Ajustes no mapeamento das entidades
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D2DD09B-8EB2-49AC-BDD9-10F3773C784C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C90B9E3-322E-47F3-84D7-F0124722A71E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{59D4C9AA-0B45-4A22-B6BD-D08E6C242389}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>US</t>
   </si>
@@ -210,6 +210,9 @@
   </si>
   <si>
     <t>Criar tela para listar os produtos femininos</t>
+  </si>
+  <si>
+    <t>3.3</t>
   </si>
 </sst>
 </file>
@@ -280,13 +283,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -639,10 +642,10 @@
       </c>
     </row>
     <row r="2" spans="1:4" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="9">
+      <c r="A2" s="10">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="5" t="s">
@@ -650,8 +653,8 @@
       </c>
     </row>
     <row r="3" spans="1:4" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="9"/>
-      <c r="B3" s="8"/>
+      <c r="A3" s="10"/>
+      <c r="B3" s="9"/>
       <c r="C3" s="5" t="s">
         <v>52</v>
       </c>
@@ -660,17 +663,17 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9"/>
-      <c r="B4" s="8"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9">
+      <c r="A5" s="10">
         <v>2</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="9" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -678,24 +681,24 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="96.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
-      <c r="B6" s="8"/>
+      <c r="A6" s="10"/>
+      <c r="B6" s="9"/>
       <c r="C6" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="9"/>
-      <c r="B7" s="8"/>
+      <c r="A7" s="10"/>
+      <c r="B7" s="9"/>
       <c r="C7" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9">
+      <c r="A8" s="10">
         <v>3</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="9" t="s">
         <v>3</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -703,44 +706,47 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
-      <c r="B9" s="8"/>
+      <c r="A9" s="10"/>
+      <c r="B9" s="9"/>
       <c r="C9" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="9"/>
-      <c r="B10" s="8"/>
+      <c r="A10" s="10"/>
+      <c r="B10" s="9"/>
       <c r="C10" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="8" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="9"/>
-      <c r="B11" s="8"/>
+      <c r="A11" s="10"/>
+      <c r="B11" s="9"/>
       <c r="C11" s="7" t="s">
         <v>54</v>
       </c>
+      <c r="D11" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="7" t="s">
+      <c r="A12" s="10"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="8" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9">
+      <c r="A13" s="10">
         <v>4</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="9" t="s">
         <v>4</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -751,31 +757,31 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="9"/>
-      <c r="B14" s="8"/>
+      <c r="A14" s="10"/>
+      <c r="B14" s="9"/>
       <c r="C14" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="9"/>
-      <c r="B15" s="8"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="9"/>
       <c r="C15" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="9"/>
-      <c r="B16" s="8"/>
+      <c r="A16" s="10"/>
+      <c r="B16" s="9"/>
       <c r="C16" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A17" s="9">
+      <c r="A17" s="10">
         <v>5</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="9" t="s">
         <v>5</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -783,17 +789,17 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="9"/>
-      <c r="B18" s="8"/>
+      <c r="A18" s="10"/>
+      <c r="B18" s="9"/>
       <c r="C18" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="9">
+      <c r="A19" s="10">
         <v>6</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -801,17 +807,17 @@
       </c>
     </row>
     <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="9"/>
-      <c r="B20" s="8"/>
+      <c r="A20" s="10"/>
+      <c r="B20" s="9"/>
       <c r="C20" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="9">
+      <c r="A21" s="10">
         <v>7</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="9" t="s">
         <v>7</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -819,8 +825,8 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="9"/>
-      <c r="B22" s="8"/>
+      <c r="A22" s="10"/>
+      <c r="B22" s="9"/>
       <c r="C22" s="2" t="s">
         <v>35</v>
       </c>
@@ -895,40 +901,40 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="9">
+      <c r="A29" s="10">
         <v>14</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="9" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="9"/>
-      <c r="B30" s="8"/>
+      <c r="A30" s="10"/>
+      <c r="B30" s="9"/>
       <c r="C30" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="9"/>
-      <c r="B31" s="8"/>
+      <c r="A31" s="10"/>
+      <c r="B31" s="9"/>
       <c r="C31" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="9"/>
-      <c r="B32" s="8"/>
+      <c r="A32" s="10"/>
+      <c r="B32" s="9"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="9"/>
-      <c r="B33" s="8"/>
+      <c r="A33" s="10"/>
+      <c r="B33" s="9"/>
     </row>
     <row r="34" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="9">
+      <c r="A34" s="10">
         <v>15</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="9" t="s">
         <v>15</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -936,42 +942,51 @@
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="9"/>
-      <c r="B35" s="8"/>
+      <c r="A35" s="10"/>
+      <c r="B35" s="9"/>
       <c r="C35" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="9"/>
-      <c r="B36" s="8"/>
+      <c r="A36" s="10"/>
+      <c r="B36" s="9"/>
       <c r="C36" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="9"/>
-      <c r="B37" s="8"/>
+      <c r="A37" s="10"/>
+      <c r="B37" s="9"/>
       <c r="C37" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="9"/>
-      <c r="B38" s="8"/>
+      <c r="A38" s="10"/>
+      <c r="B38" s="9"/>
       <c r="C38" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="9"/>
-      <c r="B39" s="8"/>
+      <c r="A39" s="10"/>
+      <c r="B39" s="9"/>
       <c r="C39" s="2" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B29:B33"/>
+    <mergeCell ref="A29:A33"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B21:B22"/>
     <mergeCell ref="B34:B39"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="A13:A16"/>
@@ -981,15 +996,6 @@
     <mergeCell ref="A34:A39"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="B8:B12"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="B29:B33"/>
-    <mergeCell ref="A29:A33"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B21:B22"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
EM-3.3 - Retornando produtos para tela home
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C90B9E3-322E-47F3-84D7-F0124722A71E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A6BBDEC-1827-47BF-ACE1-9C6004065415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{59D4C9AA-0B45-4A22-B6BD-D08E6C242389}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>US</t>
   </si>
@@ -213,6 +213,9 @@
   </si>
   <si>
     <t>3.3</t>
+  </si>
+  <si>
+    <t>1.2</t>
   </si>
 </sst>
 </file>
@@ -262,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -290,6 +293,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -642,10 +655,10 @@
       </c>
     </row>
     <row r="2" spans="1:4" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="10">
+      <c r="A2" s="12">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="11" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="5" t="s">
@@ -653,27 +666,30 @@
       </c>
     </row>
     <row r="3" spans="1:4" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="10"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="5" t="s">
+      <c r="A3" s="12"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="14" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10"/>
-      <c r="B4" s="9"/>
+      <c r="A4" s="12"/>
+      <c r="B4" s="11"/>
       <c r="C4" s="2" t="s">
         <v>21</v>
       </c>
+      <c r="D4" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="5" spans="1:4" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10">
+      <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="11" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -681,24 +697,24 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="96.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10"/>
-      <c r="B6" s="9"/>
+      <c r="A6" s="12"/>
+      <c r="B6" s="11"/>
       <c r="C6" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="10"/>
-      <c r="B7" s="9"/>
+      <c r="A7" s="12"/>
+      <c r="B7" s="11"/>
       <c r="C7" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10">
+      <c r="A8" s="12">
         <v>3</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="11" t="s">
         <v>3</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -706,15 +722,15 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="10"/>
-      <c r="B9" s="9"/>
+      <c r="A9" s="12"/>
+      <c r="B9" s="11"/>
       <c r="C9" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
-      <c r="B10" s="9"/>
+      <c r="A10" s="12"/>
+      <c r="B10" s="11"/>
       <c r="C10" s="6" t="s">
         <v>48</v>
       </c>
@@ -723,8 +739,8 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="9"/>
+      <c r="A11" s="12"/>
+      <c r="B11" s="11"/>
       <c r="C11" s="7" t="s">
         <v>54</v>
       </c>
@@ -733,8 +749,8 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
-      <c r="B12" s="9"/>
+      <c r="A12" s="12"/>
+      <c r="B12" s="11"/>
       <c r="C12" s="6" t="s">
         <v>56</v>
       </c>
@@ -743,10 +759,10 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10">
+      <c r="A13" s="12">
         <v>4</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="11" t="s">
         <v>4</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -757,31 +773,31 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="10"/>
-      <c r="B14" s="9"/>
+      <c r="A14" s="12"/>
+      <c r="B14" s="11"/>
       <c r="C14" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="10"/>
-      <c r="B15" s="9"/>
+      <c r="A15" s="12"/>
+      <c r="B15" s="11"/>
       <c r="C15" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="10"/>
-      <c r="B16" s="9"/>
+      <c r="A16" s="12"/>
+      <c r="B16" s="11"/>
       <c r="C16" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A17" s="10">
+      <c r="A17" s="12">
         <v>5</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="11" t="s">
         <v>5</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -789,17 +805,17 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="9"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="11"/>
       <c r="C18" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10">
+      <c r="A19" s="12">
         <v>6</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="11" t="s">
         <v>6</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -807,17 +823,17 @@
       </c>
     </row>
     <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
-      <c r="B20" s="9"/>
+      <c r="A20" s="12"/>
+      <c r="B20" s="11"/>
       <c r="C20" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="10">
+      <c r="A21" s="12">
         <v>7</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="11" t="s">
         <v>7</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -825,8 +841,8 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="10"/>
-      <c r="B22" s="9"/>
+      <c r="A22" s="12"/>
+      <c r="B22" s="11"/>
       <c r="C22" s="2" t="s">
         <v>35</v>
       </c>
@@ -842,11 +858,11 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="4">
+    <row r="24" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="10">
         <v>9</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="9" t="s">
         <v>9</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -901,40 +917,40 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="10">
+      <c r="A29" s="12">
         <v>14</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="11" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="10"/>
-      <c r="B30" s="9"/>
+      <c r="A30" s="12"/>
+      <c r="B30" s="11"/>
       <c r="C30" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="10"/>
-      <c r="B31" s="9"/>
+      <c r="A31" s="12"/>
+      <c r="B31" s="11"/>
       <c r="C31" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="10"/>
-      <c r="B32" s="9"/>
+      <c r="A32" s="12"/>
+      <c r="B32" s="11"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="10"/>
-      <c r="B33" s="9"/>
+      <c r="A33" s="12"/>
+      <c r="B33" s="11"/>
     </row>
     <row r="34" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="10">
+      <c r="A34" s="12">
         <v>15</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -942,42 +958,51 @@
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="10"/>
-      <c r="B35" s="9"/>
+      <c r="A35" s="12"/>
+      <c r="B35" s="11"/>
       <c r="C35" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="10"/>
-      <c r="B36" s="9"/>
+      <c r="A36" s="12"/>
+      <c r="B36" s="11"/>
       <c r="C36" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="10"/>
-      <c r="B37" s="9"/>
+      <c r="A37" s="12"/>
+      <c r="B37" s="11"/>
       <c r="C37" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="10"/>
-      <c r="B38" s="9"/>
+      <c r="A38" s="12"/>
+      <c r="B38" s="11"/>
       <c r="C38" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="10"/>
-      <c r="B39" s="9"/>
+      <c r="A39" s="12"/>
+      <c r="B39" s="11"/>
       <c r="C39" s="2" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B34:B39"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A34:A39"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="B8:B12"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="B29:B33"/>
@@ -987,15 +1012,6 @@
     <mergeCell ref="B17:B18"/>
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B34:B39"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A34:A39"/>
-    <mergeCell ref="A8:A12"/>
-    <mergeCell ref="B8:B12"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
EM-1.2 - Ajustes tela de cadastro de produtos + Rotina de cadastro no banco de dados
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A6BBDEC-1827-47BF-ACE1-9C6004065415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F477265E-031B-4129-93DD-3CC095CE78A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{59D4C9AA-0B45-4A22-B6BD-D08E6C242389}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t>US</t>
   </si>
@@ -216,6 +216,18 @@
   </si>
   <si>
     <t>1.2</t>
+  </si>
+  <si>
+    <t>Criação de rotina para cadastro de tamanhos</t>
+  </si>
+  <si>
+    <t>Página de parâmetros, para definir tipo de tamanho utilizado para cada roupa</t>
+  </si>
+  <si>
+    <t>1.4</t>
+  </si>
+  <si>
+    <t>1.3</t>
   </si>
 </sst>
 </file>
@@ -265,7 +277,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -303,6 +315,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -637,7 +655,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0855CDB-E763-4D95-8CC1-C9E4FEECBA91}">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="4"/>
@@ -654,11 +672,11 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="12">
+    <row r="2" spans="1:4" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16">
         <v>1</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="15" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="5" t="s">
@@ -666,8 +684,8 @@
       </c>
     </row>
     <row r="3" spans="1:4" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="12"/>
-      <c r="B3" s="11"/>
+      <c r="A3" s="16"/>
+      <c r="B3" s="15"/>
       <c r="C3" s="13" t="s">
         <v>52</v>
       </c>
@@ -676,8 +694,8 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12"/>
-      <c r="B4" s="11"/>
+      <c r="A4" s="16"/>
+      <c r="B4" s="15"/>
       <c r="C4" s="2" t="s">
         <v>21</v>
       </c>
@@ -686,332 +704,352 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12">
+      <c r="A5" s="12"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="16">
         <v>2</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B7" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="96.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="2" t="s">
+    <row r="8" spans="1:4" ht="96.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="16"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="12"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="2" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="16"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12">
+    <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="16">
         <v>3</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B10" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="12"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="2" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="16"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="12"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="6" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="16"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D12" s="8" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="12"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="7" t="s">
+    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="16"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D13" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="12"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="6" t="s">
+    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="16"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D14" s="8" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12">
+    <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="16">
         <v>4</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B15" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D15" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="12"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="2" t="s">
+    <row r="16" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="16"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="2" t="s">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="16"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="12"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="2" t="s">
+    <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="16"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A17" s="12">
+    <row r="19" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A19" s="16">
         <v>5</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B19" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="12"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="2" t="s">
+    <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="16"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12">
+    <row r="21" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="16">
         <v>6</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B21" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="12"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="2" t="s">
+    <row r="22" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="16"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="12">
+    <row r="23" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="16">
         <v>7</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B23" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="12"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="2" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="16"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="4">
+    <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
         <v>8</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B25" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10">
+    <row r="26" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="10">
         <v>9</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B26" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4">
+    <row r="27" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="4">
         <v>10</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D27" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A26" s="4">
+    <row r="28" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A28" s="4">
         <v>11</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B28" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="4">
+    <row r="29" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="4">
         <v>12</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B29" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="4">
+    <row r="30" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="4">
         <v>13</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B30" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="12">
+    <row r="31" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="16">
         <v>14</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B31" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="12"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="6" t="s">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="16"/>
+      <c r="B32" s="15"/>
+      <c r="C32" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="12"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="2" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="16"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="12"/>
-      <c r="B32" s="11"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="12"/>
-      <c r="B33" s="11"/>
-    </row>
-    <row r="34" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="12">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="16"/>
+      <c r="B34" s="15"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="16"/>
+      <c r="B35" s="15"/>
+    </row>
+    <row r="36" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="16">
         <v>15</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B36" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="12"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="2" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="16"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="12"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="2" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="16"/>
+      <c r="B38" s="15"/>
+      <c r="C38" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="12"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="2" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="16"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="12"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="2" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="16"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="12"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="2" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="16"/>
+      <c r="B41" s="15"/>
+      <c r="C41" s="2" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B34:B39"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B31:B35"/>
+    <mergeCell ref="A31:A35"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B15:B18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="B36:B41"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A15:A18"/>
     <mergeCell ref="A19:A20"/>
     <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A34:A39"/>
-    <mergeCell ref="A8:A12"/>
-    <mergeCell ref="B8:B12"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="B29:B33"/>
-    <mergeCell ref="A29:A33"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A36:A41"/>
+    <mergeCell ref="A10:A14"/>
+    <mergeCell ref="B10:B14"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
EM-2.3 - Rotina de inclusão de produtos por excel
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EC1936B-7C36-463C-96EE-26FF330A453D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A6E7DA0-9592-4B8E-BE65-5BC68F962409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="191">
   <si>
     <t>US</t>
   </si>
@@ -595,6 +595,9 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Criar rotina para executar em backgroud (Não sei ainda se utilizo ConcurrentDictionary ou no banco de dados)</t>
   </si>
 </sst>
 </file>
@@ -616,7 +619,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -626,6 +629,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -642,7 +651,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -654,6 +663,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1019,10 +1031,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="5">
+      <c r="A2" s="7">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1031,8 +1043,8 @@
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
       <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1041,8 +1053,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
+      <c r="A4" s="7"/>
+      <c r="B4" s="7"/>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1051,8 +1063,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
+      <c r="A5" s="7"/>
+      <c r="B5" s="7"/>
       <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1061,20 +1073,20 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="1" t="s">
+      <c r="A6" s="7"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
+      <c r="A7" s="6">
         <v>2</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -1085,8 +1097,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1097,21 +1109,24 @@
         <v>189</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="1" t="s">
+    <row r="9" spans="1:5" ht="63" x14ac:dyDescent="0.25">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="5" t="s">
         <v>124</v>
       </c>
+      <c r="E9" s="1" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="5">
+      <c r="A10" s="6">
         <v>3</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1122,8 +1137,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
       <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1132,8 +1147,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
@@ -1142,8 +1157,8 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
       <c r="C13" s="1" t="s">
         <v>21</v>
       </c>
@@ -1152,8 +1167,8 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
       <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
@@ -1162,10 +1177,10 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="5">
+      <c r="A15" s="6">
         <v>4</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C15" s="1" t="s">
@@ -1176,8 +1191,8 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
       <c r="C16" s="1" t="s">
         <v>28</v>
       </c>
@@ -1186,8 +1201,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
       <c r="C17" s="1" t="s">
         <v>29</v>
       </c>
@@ -1196,8 +1211,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
       <c r="C18" s="1" t="s">
         <v>30</v>
       </c>
@@ -1206,10 +1221,10 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="5">
+      <c r="A19" s="6">
         <v>5</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>31</v>
       </c>
       <c r="C19" s="1" t="s">
@@ -1220,8 +1235,8 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
       <c r="C20" s="1" t="s">
         <v>33</v>
       </c>
@@ -1230,10 +1245,10 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="5">
+      <c r="A21" s="6">
         <v>6</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="6" t="s">
         <v>34</v>
       </c>
       <c r="C21" s="1" t="s">
@@ -1244,8 +1259,8 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
       <c r="C22" s="1" t="s">
         <v>36</v>
       </c>
@@ -1254,10 +1269,10 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="5">
+      <c r="A23" s="6">
         <v>7</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -1268,8 +1283,8 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
       <c r="C24" s="1" t="s">
         <v>39</v>
       </c>
@@ -1334,10 +1349,10 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="5">
+      <c r="A29" s="6">
         <v>12</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="6" t="s">
         <v>49</v>
       </c>
       <c r="C29" s="1" t="s">
@@ -1348,8 +1363,8 @@
       </c>
     </row>
     <row r="30" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
+      <c r="A30" s="6"/>
+      <c r="B30" s="6"/>
       <c r="C30" s="2" t="s">
         <v>135</v>
       </c>
@@ -1372,48 +1387,48 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="6">
+      <c r="A32" s="7">
         <v>14</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="7" t="s">
         <v>53</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="6"/>
-      <c r="B33" s="6"/>
+      <c r="A33" s="7"/>
+      <c r="B33" s="7"/>
       <c r="C33" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D33" s="3"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="6"/>
-      <c r="B34" s="6"/>
+      <c r="A34" s="7"/>
+      <c r="B34" s="7"/>
       <c r="C34" s="3" t="s">
         <v>55</v>
       </c>
       <c r="D34" s="3"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="6"/>
-      <c r="B35" s="6"/>
+      <c r="A35" s="7"/>
+      <c r="B35" s="7"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="6"/>
-      <c r="B36" s="6"/>
+      <c r="A36" s="7"/>
+      <c r="B36" s="7"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="5">
+      <c r="A37" s="6">
         <v>15</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="6" t="s">
         <v>56</v>
       </c>
       <c r="C37" s="1" t="s">
@@ -1424,8 +1439,8 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
+      <c r="A38" s="6"/>
+      <c r="B38" s="6"/>
       <c r="C38" s="1" t="s">
         <v>58</v>
       </c>
@@ -1434,8 +1449,8 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
+      <c r="A39" s="6"/>
+      <c r="B39" s="6"/>
       <c r="C39" s="1" t="s">
         <v>59</v>
       </c>
@@ -1444,8 +1459,8 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
+      <c r="A40" s="6"/>
+      <c r="B40" s="6"/>
       <c r="C40" s="1" t="s">
         <v>60</v>
       </c>
@@ -1454,8 +1469,8 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
+      <c r="A41" s="6"/>
+      <c r="B41" s="6"/>
       <c r="C41" s="1" t="s">
         <v>61</v>
       </c>
@@ -1464,8 +1479,8 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="5"/>
-      <c r="B42" s="5"/>
+      <c r="A42" s="6"/>
+      <c r="B42" s="6"/>
       <c r="C42" s="1" t="s">
         <v>62</v>
       </c>
@@ -1474,10 +1489,10 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="5">
+      <c r="A43" s="6">
         <v>16</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="6" t="s">
         <v>74</v>
       </c>
       <c r="C43" s="1" t="s">
@@ -1488,8 +1503,8 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5"/>
+      <c r="A44" s="6"/>
+      <c r="B44" s="6"/>
       <c r="C44" s="1" t="s">
         <v>64</v>
       </c>
@@ -1498,8 +1513,8 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="5"/>
-      <c r="B45" s="5"/>
+      <c r="A45" s="6"/>
+      <c r="B45" s="6"/>
       <c r="C45" s="1" t="s">
         <v>65</v>
       </c>
@@ -1508,8 +1523,8 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="5"/>
-      <c r="B46" s="5"/>
+      <c r="A46" s="6"/>
+      <c r="B46" s="6"/>
       <c r="C46" s="1" t="s">
         <v>66</v>
       </c>
@@ -1518,8 +1533,8 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5"/>
+      <c r="A47" s="6"/>
+      <c r="B47" s="6"/>
       <c r="C47" s="1" t="s">
         <v>69</v>
       </c>
@@ -1528,8 +1543,8 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="5"/>
-      <c r="B48" s="5"/>
+      <c r="A48" s="6"/>
+      <c r="B48" s="6"/>
       <c r="C48" s="1" t="s">
         <v>73</v>
       </c>
@@ -1538,8 +1553,8 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="5"/>
-      <c r="B49" s="5"/>
+      <c r="A49" s="6"/>
+      <c r="B49" s="6"/>
       <c r="C49" s="1" t="s">
         <v>75</v>
       </c>
@@ -1548,8 +1563,8 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="5"/>
-      <c r="B50" s="5"/>
+      <c r="A50" s="6"/>
+      <c r="B50" s="6"/>
       <c r="C50" s="1" t="s">
         <v>76</v>
       </c>
@@ -1558,8 +1573,8 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="5"/>
-      <c r="B51" s="5"/>
+      <c r="A51" s="6"/>
+      <c r="B51" s="6"/>
       <c r="C51" s="1" t="s">
         <v>77</v>
       </c>
@@ -1568,10 +1583,10 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="5">
+      <c r="A52" s="6">
         <v>17</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B52" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C52" s="1" t="s">
@@ -1582,8 +1597,8 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="5"/>
-      <c r="B53" s="5"/>
+      <c r="A53" s="6"/>
+      <c r="B53" s="6"/>
       <c r="C53" s="1" t="s">
         <v>80</v>
       </c>
@@ -1592,8 +1607,8 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="5"/>
-      <c r="B54" s="5"/>
+      <c r="A54" s="6"/>
+      <c r="B54" s="6"/>
       <c r="C54" s="1" t="s">
         <v>81</v>
       </c>
@@ -1602,8 +1617,8 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="5"/>
-      <c r="B55" s="5"/>
+      <c r="A55" s="6"/>
+      <c r="B55" s="6"/>
       <c r="C55" s="1" t="s">
         <v>82</v>
       </c>
@@ -1612,10 +1627,10 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="5">
+      <c r="A56" s="6">
         <v>18</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="B56" s="6" t="s">
         <v>83</v>
       </c>
       <c r="C56" s="1" t="s">
@@ -1626,8 +1641,8 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="5"/>
-      <c r="B57" s="5"/>
+      <c r="A57" s="6"/>
+      <c r="B57" s="6"/>
       <c r="C57" s="1" t="s">
         <v>85</v>
       </c>
@@ -1636,8 +1651,8 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="5"/>
-      <c r="B58" s="5"/>
+      <c r="A58" s="6"/>
+      <c r="B58" s="6"/>
       <c r="C58" s="1" t="s">
         <v>86</v>
       </c>
@@ -1646,8 +1661,8 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="5"/>
-      <c r="B59" s="5"/>
+      <c r="A59" s="6"/>
+      <c r="B59" s="6"/>
       <c r="C59" s="1" t="s">
         <v>87</v>
       </c>
@@ -1656,10 +1671,10 @@
       </c>
     </row>
     <row r="60" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A60" s="5">
+      <c r="A60" s="6">
         <v>19</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="B60" s="6" t="s">
         <v>88</v>
       </c>
       <c r="C60" s="1" t="s">
@@ -1670,8 +1685,8 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="5"/>
-      <c r="B61" s="5"/>
+      <c r="A61" s="6"/>
+      <c r="B61" s="6"/>
       <c r="C61" s="1" t="s">
         <v>90</v>
       </c>
@@ -1680,8 +1695,8 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="5"/>
-      <c r="B62" s="5"/>
+      <c r="A62" s="6"/>
+      <c r="B62" s="6"/>
       <c r="C62" s="1" t="s">
         <v>91</v>
       </c>
@@ -1690,8 +1705,8 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="5"/>
-      <c r="B63" s="5"/>
+      <c r="A63" s="6"/>
+      <c r="B63" s="6"/>
       <c r="C63" s="1" t="s">
         <v>92</v>
       </c>
@@ -1700,10 +1715,10 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="5">
+      <c r="A64" s="6">
         <v>20</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="B64" s="6" t="s">
         <v>93</v>
       </c>
       <c r="C64" s="1" t="s">
@@ -1714,8 +1729,8 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="5"/>
-      <c r="B65" s="5"/>
+      <c r="A65" s="6"/>
+      <c r="B65" s="6"/>
       <c r="C65" s="1" t="s">
         <v>95</v>
       </c>
@@ -1724,8 +1739,8 @@
       </c>
     </row>
     <row r="66" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A66" s="5"/>
-      <c r="B66" s="5"/>
+      <c r="A66" s="6"/>
+      <c r="B66" s="6"/>
       <c r="C66" s="1" t="s">
         <v>96</v>
       </c>
@@ -1734,8 +1749,8 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="5"/>
-      <c r="B67" s="5"/>
+      <c r="A67" s="6"/>
+      <c r="B67" s="6"/>
       <c r="C67" s="1" t="s">
         <v>97</v>
       </c>
@@ -1744,10 +1759,10 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="5">
+      <c r="A68" s="6">
         <v>21</v>
       </c>
-      <c r="B68" s="5" t="s">
+      <c r="B68" s="6" t="s">
         <v>98</v>
       </c>
       <c r="C68" s="1" t="s">
@@ -1758,8 +1773,8 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="5"/>
-      <c r="B69" s="5"/>
+      <c r="A69" s="6"/>
+      <c r="B69" s="6"/>
       <c r="C69" s="1" t="s">
         <v>100</v>
       </c>
@@ -1768,8 +1783,8 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="5"/>
-      <c r="B70" s="5"/>
+      <c r="A70" s="6"/>
+      <c r="B70" s="6"/>
       <c r="C70" s="1" t="s">
         <v>101</v>
       </c>
@@ -1778,8 +1793,8 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="5"/>
-      <c r="B71" s="5"/>
+      <c r="A71" s="6"/>
+      <c r="B71" s="6"/>
       <c r="C71" s="1" t="s">
         <v>102</v>
       </c>
@@ -1788,10 +1803,10 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="5">
+      <c r="A72" s="6">
         <v>22</v>
       </c>
-      <c r="B72" s="5" t="s">
+      <c r="B72" s="6" t="s">
         <v>103</v>
       </c>
       <c r="C72" s="1" t="s">
@@ -1802,8 +1817,8 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="5"/>
-      <c r="B73" s="5"/>
+      <c r="A73" s="6"/>
+      <c r="B73" s="6"/>
       <c r="C73" s="1" t="s">
         <v>105</v>
       </c>
@@ -1812,8 +1827,8 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="5"/>
-      <c r="B74" s="5"/>
+      <c r="A74" s="6"/>
+      <c r="B74" s="6"/>
       <c r="C74" s="1" t="s">
         <v>106</v>
       </c>
@@ -1822,8 +1837,8 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="5"/>
-      <c r="B75" s="5"/>
+      <c r="A75" s="6"/>
+      <c r="B75" s="6"/>
       <c r="C75" s="1" t="s">
         <v>107</v>
       </c>
@@ -1832,8 +1847,8 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="5"/>
-      <c r="B76" s="5"/>
+      <c r="A76" s="6"/>
+      <c r="B76" s="6"/>
       <c r="C76" s="1" t="s">
         <v>108</v>
       </c>
@@ -1842,10 +1857,10 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="5">
+      <c r="A77" s="6">
         <v>23</v>
       </c>
-      <c r="B77" s="5" t="s">
+      <c r="B77" s="6" t="s">
         <v>109</v>
       </c>
       <c r="C77" s="1" t="s">
@@ -1856,8 +1871,8 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="5"/>
-      <c r="B78" s="5"/>
+      <c r="A78" s="6"/>
+      <c r="B78" s="6"/>
       <c r="C78" s="1" t="s">
         <v>111</v>
       </c>
@@ -1866,8 +1881,8 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="5"/>
-      <c r="B79" s="5"/>
+      <c r="A79" s="6"/>
+      <c r="B79" s="6"/>
       <c r="C79" s="1" t="s">
         <v>112</v>
       </c>
@@ -1876,10 +1891,10 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="5">
+      <c r="A80" s="6">
         <v>24</v>
       </c>
-      <c r="B80" s="5" t="s">
+      <c r="B80" s="6" t="s">
         <v>113</v>
       </c>
       <c r="C80" s="1" t="s">
@@ -1890,8 +1905,8 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="5"/>
-      <c r="B81" s="5"/>
+      <c r="A81" s="6"/>
+      <c r="B81" s="6"/>
       <c r="C81" s="1" t="s">
         <v>115</v>
       </c>
@@ -1900,8 +1915,8 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="5"/>
-      <c r="B82" s="5"/>
+      <c r="A82" s="6"/>
+      <c r="B82" s="6"/>
       <c r="C82" s="1" t="s">
         <v>116</v>
       </c>
@@ -1910,10 +1925,10 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="5">
+      <c r="A83" s="6">
         <v>25</v>
       </c>
-      <c r="B83" s="5" t="s">
+      <c r="B83" s="6" t="s">
         <v>117</v>
       </c>
       <c r="C83" s="1" t="s">
@@ -1924,8 +1939,8 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="5"/>
-      <c r="B84" s="5"/>
+      <c r="A84" s="6"/>
+      <c r="B84" s="6"/>
       <c r="C84" s="1" t="s">
         <v>119</v>
       </c>
@@ -1934,8 +1949,8 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="5"/>
-      <c r="B85" s="5"/>
+      <c r="A85" s="6"/>
+      <c r="B85" s="6"/>
       <c r="C85" s="1" t="s">
         <v>120</v>
       </c>
@@ -1944,8 +1959,8 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="5"/>
-      <c r="B86" s="5"/>
+      <c r="A86" s="6"/>
+      <c r="B86" s="6"/>
       <c r="C86" s="1" t="s">
         <v>121</v>
       </c>

</xml_diff>

<commit_message>
EM-4.5,4.6,4.7 - Rotina de cadastro, login, autorização
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A6E7DA0-9592-4B8E-BE65-5BC68F962409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9F7B12F-B767-476A-BA02-0743C0D2AD44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
   <si>
     <t>US</t>
   </si>
@@ -597,7 +597,22 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>Criar rotina para executar em backgroud (Não sei ainda se utilizo ConcurrentDictionary ou no banco de dados)</t>
+    <t>Criar diagrama de usuários e papéis</t>
+  </si>
+  <si>
+    <t>4.5</t>
+  </si>
+  <si>
+    <t>Criar telas de login e cadastro</t>
+  </si>
+  <si>
+    <t>4.6</t>
+  </si>
+  <si>
+    <t>4.7</t>
+  </si>
+  <si>
+    <t>Criar rotina para login</t>
   </si>
 </sst>
 </file>
@@ -651,7 +666,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -666,6 +681,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1008,7 +1035,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E86"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
@@ -1031,10 +1058,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="7">
+      <c r="A2" s="11">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="11" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1043,8 +1070,8 @@
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
+      <c r="A3" s="11"/>
+      <c r="B3" s="11"/>
       <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1053,8 +1080,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="11"/>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1063,8 +1090,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="11"/>
       <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1073,8 +1100,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
+      <c r="A6" s="11"/>
+      <c r="B6" s="11"/>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1083,22 +1110,22 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="6">
+      <c r="A7" s="10">
         <v>2</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="7" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1109,24 +1136,22 @@
         <v>189</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="63" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="5" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>190</v>
-      </c>
+      <c r="E9" s="8"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
+      <c r="A10" s="10">
         <v>3</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1137,8 +1162,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
       <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1147,8 +1172,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
@@ -1157,18 +1182,18 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="1" t="s">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="8" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
       <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
@@ -1176,845 +1201,875 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="6">
+    <row r="15" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10">
         <v>4</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D18" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="1" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D19" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="6"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="1" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D20" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="6"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="1" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="6">
+    <row r="22" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="10">
         <v>5</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B22" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D22" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="6"/>
-      <c r="B20" s="6"/>
-      <c r="C20" s="1" t="s">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D23" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="6">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="10">
         <v>6</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B24" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C24" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D24" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="6"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="1" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="6">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="10">
         <v>7</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B26" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D26" s="1" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="6"/>
-      <c r="B24" s="6"/>
-      <c r="C24" s="1" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="10"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>130</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
-        <v>8</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
-        <v>9</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
-        <v>10</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="6">
-        <v>12</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>49</v>
+        <v>131</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>9</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="6"/>
-      <c r="B30" s="6"/>
-      <c r="C30" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>10</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
+        <v>11</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="10">
+        <v>12</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="10"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
         <v>13</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C34" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D34" s="1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="7">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="11">
         <v>14</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B35" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="7"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D33" s="3"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="7"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D34" s="3"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="7"/>
-      <c r="B36" s="7"/>
-      <c r="C36" s="3"/>
+      <c r="A36" s="11"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="3" t="s">
+        <v>54</v>
+      </c>
       <c r="D36" s="3"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="6">
+      <c r="A37" s="11"/>
+      <c r="B37" s="11"/>
+      <c r="C37" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D37" s="3"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="11"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="11"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="10">
         <v>15</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B40" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C40" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D40" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="6"/>
-      <c r="B38" s="6"/>
-      <c r="C38" s="1" t="s">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="10"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D41" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="6"/>
-      <c r="B39" s="6"/>
-      <c r="C39" s="1" t="s">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="10"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="6"/>
-      <c r="B40" s="6"/>
-      <c r="C40" s="1" t="s">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="10"/>
+      <c r="B43" s="10"/>
+      <c r="C43" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D43" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="6"/>
-      <c r="B41" s="6"/>
-      <c r="C41" s="1" t="s">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="10"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="D44" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="6"/>
-      <c r="B42" s="6"/>
-      <c r="C42" s="1" t="s">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="10"/>
+      <c r="B45" s="10"/>
+      <c r="C45" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="D45" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="6">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="10">
         <v>16</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B46" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C46" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="D46" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="6"/>
-      <c r="B44" s="6"/>
-      <c r="C44" s="1" t="s">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="10"/>
+      <c r="B47" s="10"/>
+      <c r="C47" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="D47" s="1" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="6"/>
-      <c r="B45" s="6"/>
-      <c r="C45" s="1" t="s">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="10"/>
+      <c r="B48" s="10"/>
+      <c r="C48" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="D48" s="2" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="6"/>
-      <c r="B46" s="6"/>
-      <c r="C46" s="1" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="10"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D46" s="2" t="s">
+      <c r="D49" s="2" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="6"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="1" t="s">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="10"/>
+      <c r="B50" s="10"/>
+      <c r="C50" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D47" s="2" t="s">
+      <c r="D50" s="2" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="6"/>
-      <c r="B48" s="6"/>
-      <c r="C48" s="1" t="s">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="10"/>
+      <c r="B51" s="10"/>
+      <c r="C51" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="D51" s="2" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="6"/>
-      <c r="B49" s="6"/>
-      <c r="C49" s="1" t="s">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="10"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D49" s="2" t="s">
+      <c r="D52" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="6"/>
-      <c r="B50" s="6"/>
-      <c r="C50" s="1" t="s">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="10"/>
+      <c r="B53" s="10"/>
+      <c r="C53" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D50" s="2" t="s">
+      <c r="D53" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="6"/>
-      <c r="B51" s="6"/>
-      <c r="C51" s="1" t="s">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="10"/>
+      <c r="B54" s="10"/>
+      <c r="C54" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D51" s="2" t="s">
+      <c r="D54" s="2" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="6">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="10">
         <v>17</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B55" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="C55" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D52" s="1" t="s">
+      <c r="D55" s="1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="6"/>
-      <c r="B53" s="6"/>
-      <c r="C53" s="1" t="s">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="10"/>
+      <c r="B56" s="10"/>
+      <c r="C56" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D53" s="1" t="s">
+      <c r="D56" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="6"/>
-      <c r="B54" s="6"/>
-      <c r="C54" s="1" t="s">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="10"/>
+      <c r="B57" s="10"/>
+      <c r="C57" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D54" s="2" t="s">
+      <c r="D57" s="2" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="6"/>
-      <c r="B55" s="6"/>
-      <c r="C55" s="1" t="s">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="10"/>
+      <c r="B58" s="10"/>
+      <c r="C58" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D55" s="2" t="s">
+      <c r="D58" s="2" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="6">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="10">
         <v>18</v>
       </c>
-      <c r="B56" s="6" t="s">
+      <c r="B59" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C59" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D56" s="1" t="s">
+      <c r="D59" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="6"/>
-      <c r="B57" s="6"/>
-      <c r="C57" s="1" t="s">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="10"/>
+      <c r="B60" s="10"/>
+      <c r="C60" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D57" s="1" t="s">
+      <c r="D60" s="1" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="6"/>
-      <c r="B58" s="6"/>
-      <c r="C58" s="1" t="s">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="10"/>
+      <c r="B61" s="10"/>
+      <c r="C61" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D58" s="2" t="s">
+      <c r="D61" s="2" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="6"/>
-      <c r="B59" s="6"/>
-      <c r="C59" s="1" t="s">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="10"/>
+      <c r="B62" s="10"/>
+      <c r="C62" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D59" s="2" t="s">
+      <c r="D62" s="2" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A60" s="6">
+    <row r="63" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A63" s="10">
         <v>19</v>
       </c>
-      <c r="B60" s="6" t="s">
+      <c r="B63" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="C60" s="1" t="s">
+      <c r="C63" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D60" s="1" t="s">
+      <c r="D63" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="6"/>
-      <c r="B61" s="6"/>
-      <c r="C61" s="1" t="s">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="10"/>
+      <c r="B64" s="10"/>
+      <c r="C64" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D61" s="1" t="s">
+      <c r="D64" s="1" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="6"/>
-      <c r="B62" s="6"/>
-      <c r="C62" s="1" t="s">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="10"/>
+      <c r="B65" s="10"/>
+      <c r="C65" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="D65" s="2" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="6"/>
-      <c r="B63" s="6"/>
-      <c r="C63" s="1" t="s">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="10"/>
+      <c r="B66" s="10"/>
+      <c r="C66" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D63" s="2" t="s">
+      <c r="D66" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="6">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="10">
         <v>20</v>
       </c>
-      <c r="B64" s="6" t="s">
+      <c r="B67" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="C64" s="1" t="s">
+      <c r="C67" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D64" s="1" t="s">
+      <c r="D67" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="6"/>
-      <c r="B65" s="6"/>
-      <c r="C65" s="1" t="s">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="10"/>
+      <c r="B68" s="10"/>
+      <c r="C68" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D65" s="1" t="s">
+      <c r="D68" s="1" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="66" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A66" s="6"/>
-      <c r="B66" s="6"/>
-      <c r="C66" s="1" t="s">
+    <row r="69" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A69" s="10"/>
+      <c r="B69" s="10"/>
+      <c r="C69" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D66" s="2" t="s">
+      <c r="D69" s="2" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="6"/>
-      <c r="B67" s="6"/>
-      <c r="C67" s="1" t="s">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="10"/>
+      <c r="B70" s="10"/>
+      <c r="C70" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D67" s="2" t="s">
+      <c r="D70" s="2" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="6">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="10">
         <v>21</v>
       </c>
-      <c r="B68" s="6" t="s">
+      <c r="B71" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="C68" s="1" t="s">
+      <c r="C71" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D68" s="1" t="s">
+      <c r="D71" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="6"/>
-      <c r="B69" s="6"/>
-      <c r="C69" s="1" t="s">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="10"/>
+      <c r="B72" s="10"/>
+      <c r="C72" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D69" s="1" t="s">
+      <c r="D72" s="1" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="6"/>
-      <c r="B70" s="6"/>
-      <c r="C70" s="1" t="s">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="10"/>
+      <c r="B73" s="10"/>
+      <c r="C73" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D70" s="2" t="s">
+      <c r="D73" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="6"/>
-      <c r="B71" s="6"/>
-      <c r="C71" s="1" t="s">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="10"/>
+      <c r="B74" s="10"/>
+      <c r="C74" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D71" s="2" t="s">
+      <c r="D74" s="2" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="6">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="10">
         <v>22</v>
       </c>
-      <c r="B72" s="6" t="s">
+      <c r="B75" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C72" s="1" t="s">
+      <c r="C75" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D72" s="1" t="s">
+      <c r="D75" s="1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="6"/>
-      <c r="B73" s="6"/>
-      <c r="C73" s="1" t="s">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="10"/>
+      <c r="B76" s="10"/>
+      <c r="C76" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D73" s="1" t="s">
+      <c r="D76" s="1" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="6"/>
-      <c r="B74" s="6"/>
-      <c r="C74" s="1" t="s">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="10"/>
+      <c r="B77" s="10"/>
+      <c r="C77" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D74" s="2" t="s">
+      <c r="D77" s="2" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="6"/>
-      <c r="B75" s="6"/>
-      <c r="C75" s="1" t="s">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="10"/>
+      <c r="B78" s="10"/>
+      <c r="C78" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D75" s="2" t="s">
+      <c r="D78" s="2" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="6"/>
-      <c r="B76" s="6"/>
-      <c r="C76" s="1" t="s">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="10"/>
+      <c r="B79" s="10"/>
+      <c r="C79" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="D76" s="2" t="s">
+      <c r="D79" s="2" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="6">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="10">
         <v>23</v>
       </c>
-      <c r="B77" s="6" t="s">
+      <c r="B80" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="C77" s="1" t="s">
+      <c r="C80" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D77" s="1" t="s">
+      <c r="D80" s="1" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="6"/>
-      <c r="B78" s="6"/>
-      <c r="C78" s="1" t="s">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="10"/>
+      <c r="B81" s="10"/>
+      <c r="C81" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D78" s="1" t="s">
+      <c r="D81" s="1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="6"/>
-      <c r="B79" s="6"/>
-      <c r="C79" s="1" t="s">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" s="10"/>
+      <c r="B82" s="10"/>
+      <c r="C82" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D79" s="1" t="s">
+      <c r="D82" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="6">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="10">
         <v>24</v>
       </c>
-      <c r="B80" s="6" t="s">
+      <c r="B83" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="C80" s="1" t="s">
+      <c r="C83" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D80" s="1" t="s">
+      <c r="D83" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="6"/>
-      <c r="B81" s="6"/>
-      <c r="C81" s="1" t="s">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="10"/>
+      <c r="B84" s="10"/>
+      <c r="C84" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D81" s="1" t="s">
+      <c r="D84" s="1" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="6"/>
-      <c r="B82" s="6"/>
-      <c r="C82" s="1" t="s">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="10"/>
+      <c r="B85" s="10"/>
+      <c r="C85" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D82" s="1" t="s">
+      <c r="D85" s="1" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="6">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="10">
         <v>25</v>
       </c>
-      <c r="B83" s="6" t="s">
+      <c r="B86" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C83" s="1" t="s">
+      <c r="C86" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D83" s="1" t="s">
+      <c r="D86" s="1" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="6"/>
-      <c r="B84" s="6"/>
-      <c r="C84" s="1" t="s">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="10"/>
+      <c r="B87" s="10"/>
+      <c r="C87" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D84" s="1" t="s">
+      <c r="D87" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="6"/>
-      <c r="B85" s="6"/>
-      <c r="C85" s="1" t="s">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="10"/>
+      <c r="B88" s="10"/>
+      <c r="C88" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D85" s="1" t="s">
+      <c r="D88" s="1" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="6"/>
-      <c r="B86" s="6"/>
-      <c r="C86" s="1" t="s">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="10"/>
+      <c r="B89" s="10"/>
+      <c r="C89" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D86" s="1" t="s">
+      <c r="D89" s="1" t="s">
         <v>187</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="B80:B82"/>
-    <mergeCell ref="B83:B86"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="A83:A86"/>
-    <mergeCell ref="B68:B71"/>
-    <mergeCell ref="A68:A71"/>
-    <mergeCell ref="B72:B76"/>
-    <mergeCell ref="A72:A76"/>
-    <mergeCell ref="A77:A79"/>
-    <mergeCell ref="B77:B79"/>
-    <mergeCell ref="B56:B59"/>
-    <mergeCell ref="A56:A59"/>
-    <mergeCell ref="B60:B63"/>
-    <mergeCell ref="A60:A63"/>
-    <mergeCell ref="B64:B67"/>
-    <mergeCell ref="A64:A67"/>
-    <mergeCell ref="B43:B51"/>
-    <mergeCell ref="A43:A51"/>
-    <mergeCell ref="B52:B55"/>
-    <mergeCell ref="A52:A55"/>
-    <mergeCell ref="B37:B42"/>
-    <mergeCell ref="A37:A42"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="A32:A36"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="B15:B18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A10:A14"/>
     <mergeCell ref="B2:B6"/>
     <mergeCell ref="A2:A6"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="A32:A33"/>
     <mergeCell ref="B10:B14"/>
+    <mergeCell ref="A15:A21"/>
+    <mergeCell ref="B15:B21"/>
+    <mergeCell ref="B35:B39"/>
+    <mergeCell ref="A35:A39"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A10:A14"/>
+    <mergeCell ref="B46:B54"/>
+    <mergeCell ref="A46:A54"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="B40:B45"/>
+    <mergeCell ref="A40:A45"/>
+    <mergeCell ref="B59:B62"/>
+    <mergeCell ref="A59:A62"/>
+    <mergeCell ref="B63:B66"/>
+    <mergeCell ref="A63:A66"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="A67:A70"/>
+    <mergeCell ref="B83:B85"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="A83:A85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="B71:B74"/>
+    <mergeCell ref="A71:A74"/>
+    <mergeCell ref="B75:B79"/>
+    <mergeCell ref="A75:A79"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="B80:B82"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D2 A15:D15 B3:D6 C43 A52:C52 C44:C45 C49:C51 A56:C56 C54:C55 A60:C60 C58:C59 A64:C64 C62:C63 A68:C68 C66:C67 A72:C72 C70:C71 A77:C77 C74:C76 A80:C80 C79 A83:C83 C82 C86 A7:C7 A8:C8 A9:C9 A10:C10 A11:C11 A12:C12 A13:C13 A14:C14 A27:D27 A16:C16 A17:C17 A18:C18 A19:C19 A20:C20 A21:C21 A22:C22 A23:C23 A24:C24 A25:C25 A26:C26 A32:D36 A28:C28 A29:C29 A31:C31 A42:C42 A37:C37 A38:C38 A39:C39 A40:C40 A41:C41 C47 C48 C46 C53 C57 C61 C65 C69 C73 C78 C81 C84 C85" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D2 C18:D18 B3:D6 C46 A55:C55 C47:C48 C52:C54 A59:C59 C57:C58 A63:C63 C61:C62 A67:C67 C65:C66 A71:C71 C69:C70 A75:C75 C73:C74 A80:C80 C77:C79 A83:C83 C82 A86:C86 C85 C89 A7:C7 A8:C8 A9:C9 A10:C10 A11:C11 A12:C12 A13:C13 A14:C14 A30:D30 C19 C20 C21 A22:C22 A23:C23 A24:C24 A25:C25 A26:C26 A27:C27 A28:C28 A29:C29 A35:D39 A31:C31 A32:C32 A34:C34 A45:C45 A40:C40 A41:C41 A42:C42 A43:C43 A44:C44 C50 C51 C49 C56 C60 C64 C68 C72 C76 C81 C84 C87 C88" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
EM-4.1,4.2 - Implementado carrinho de compras
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9F7B12F-B767-476A-BA02-0743C0D2AD44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98314F05-207A-426E-9DEC-D7F926ABC9DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -114,9 +114,6 @@
     <t>Criar rotina para armazenar os produtos selecionados em cache (REDIS)</t>
   </si>
   <si>
-    <t>Criar tela para finalização da compra</t>
-  </si>
-  <si>
     <t>Criar rotina para pagamento, integração com meios de pagamentos</t>
   </si>
   <si>
@@ -613,6 +610,9 @@
   </si>
   <si>
     <t>Criar rotina para login</t>
+  </si>
+  <si>
+    <t>Criar rotina para finalização da compra</t>
   </si>
 </sst>
 </file>
@@ -634,7 +634,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -644,12 +644,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -680,9 +674,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -695,10 +686,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1054,14 +1048,14 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="11">
+      <c r="A2" s="10">
         <v>1</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1070,8 +1064,8 @@
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
+      <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
       <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1080,8 +1074,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="11"/>
-      <c r="B4" s="11"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1090,8 +1084,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="11"/>
-      <c r="B5" s="11"/>
+      <c r="A5" s="10"/>
+      <c r="B5" s="10"/>
       <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1100,8 +1094,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="11"/>
-      <c r="B6" s="11"/>
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1110,48 +1104,48 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="10">
+      <c r="A7" s="11">
         <v>2</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>122</v>
+      <c r="D7" s="6" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
-      <c r="B8" s="10"/>
+      <c r="A8" s="11"/>
+      <c r="B8" s="11"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="11"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="E9" s="8"/>
+      <c r="E9" s="7"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="10">
+      <c r="A10" s="11">
         <v>3</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1162,8 +1156,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
       <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1172,8 +1166,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="11"/>
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
@@ -1182,169 +1176,169 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="8" t="s">
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="8" t="s">
-        <v>67</v>
+      <c r="D13" s="7" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
       <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="11">
         <v>4</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="D15" s="9" t="s">
+    </row>
+    <row r="16" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="8" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="9" t="s">
+      <c r="D16" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="D16" s="9" t="s">
+    </row>
+    <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="17" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="9" t="s">
+    <row r="18" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="D17" s="9" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="1" t="s">
+      <c r="D20" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="1" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="11"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="10"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="1" t="s">
+    <row r="22" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="11">
+        <v>5</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="10">
-        <v>5</v>
-      </c>
-      <c r="B22" s="10" t="s">
+      <c r="C22" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="D22" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="11"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D23" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="1" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="11">
+        <v>6</v>
+      </c>
+      <c r="B24" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="C24" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="10">
-        <v>6</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C24" s="1" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="11"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="10"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="1" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="11">
+        <v>7</v>
+      </c>
+      <c r="B26" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="C26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="10">
-        <v>7</v>
-      </c>
-      <c r="B26" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C26" s="1" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="11"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>129</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="10"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
@@ -1352,13 +1346,13 @@
         <v>8</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="D28" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
@@ -1366,13 +1360,13 @@
         <v>9</v>
       </c>
       <c r="B29" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="D29" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
@@ -1380,13 +1374,13 @@
         <v>10</v>
       </c>
       <c r="B30" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="D30" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
@@ -1394,37 +1388,37 @@
         <v>11</v>
       </c>
       <c r="B31" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="D31" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="11">
+        <v>12</v>
+      </c>
+      <c r="B32" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="C32" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="10">
-        <v>12</v>
-      </c>
-      <c r="B32" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D32" s="1" t="s">
+    <row r="33" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="11"/>
+      <c r="B33" s="11"/>
+      <c r="C33" s="2" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="2" t="s">
+      <c r="D33" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
@@ -1432,606 +1426,621 @@
         <v>13</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="D34" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="10">
+        <v>14</v>
+      </c>
+      <c r="B35" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="11">
-        <v>14</v>
-      </c>
-      <c r="B35" s="11" t="s">
-        <v>53</v>
       </c>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="11"/>
-      <c r="B36" s="11"/>
+      <c r="A36" s="10"/>
+      <c r="B36" s="10"/>
       <c r="C36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D36" s="3"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="10"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D36" s="3"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="11"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="3" t="s">
-        <v>55</v>
-      </c>
       <c r="D37" s="3"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="11"/>
-      <c r="B38" s="11"/>
+      <c r="A38" s="10"/>
+      <c r="B38" s="10"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="11"/>
-      <c r="B39" s="11"/>
+      <c r="A39" s="10"/>
+      <c r="B39" s="10"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="10">
+      <c r="A40" s="11">
         <v>15</v>
       </c>
-      <c r="B40" s="10" t="s">
+      <c r="B40" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="D40" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="11"/>
+      <c r="B41" s="11"/>
+      <c r="C41" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D41" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="10"/>
-      <c r="B41" s="10"/>
-      <c r="C41" s="1" t="s">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="11"/>
+      <c r="B42" s="11"/>
+      <c r="C42" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="10"/>
-      <c r="B42" s="10"/>
-      <c r="C42" s="1" t="s">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="11"/>
+      <c r="B43" s="11"/>
+      <c r="C43" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="D43" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="10"/>
-      <c r="B43" s="10"/>
-      <c r="C43" s="1" t="s">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="11"/>
+      <c r="B44" s="11"/>
+      <c r="C44" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="D44" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="10"/>
-      <c r="B44" s="10"/>
-      <c r="C44" s="1" t="s">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="11"/>
+      <c r="B45" s="11"/>
+      <c r="C45" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="D45" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="10"/>
-      <c r="B45" s="10"/>
-      <c r="C45" s="1" t="s">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="11">
+        <v>16</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C46" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="D46" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="10">
-        <v>16</v>
-      </c>
-      <c r="B46" s="10" t="s">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="11"/>
+      <c r="B47" s="11"/>
+      <c r="C47" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="11"/>
+      <c r="B48" s="11"/>
+      <c r="C48" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="11"/>
+      <c r="B49" s="11"/>
+      <c r="C49" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="11"/>
+      <c r="B50" s="11"/>
+      <c r="C50" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="11"/>
+      <c r="B51" s="11"/>
+      <c r="C51" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="11"/>
+      <c r="B52" s="11"/>
+      <c r="C52" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C46" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="10"/>
-      <c r="B47" s="10"/>
-      <c r="C47" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="10"/>
-      <c r="B48" s="10"/>
-      <c r="C48" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="10"/>
-      <c r="B49" s="10"/>
-      <c r="C49" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="10"/>
-      <c r="B50" s="10"/>
-      <c r="C50" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="10"/>
-      <c r="B51" s="10"/>
-      <c r="C51" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D51" s="2" t="s">
+      <c r="D52" s="2" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="10"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="1" t="s">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="11"/>
+      <c r="B53" s="11"/>
+      <c r="C53" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D52" s="2" t="s">
+      <c r="D53" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="10"/>
-      <c r="B53" s="10"/>
-      <c r="C53" s="1" t="s">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="11"/>
+      <c r="B54" s="11"/>
+      <c r="C54" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D53" s="2" t="s">
+      <c r="D54" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="10"/>
-      <c r="B54" s="10"/>
-      <c r="C54" s="1" t="s">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="11">
+        <v>17</v>
+      </c>
+      <c r="B55" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="D54" s="2" t="s">
+      <c r="C55" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D55" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="10">
-        <v>17</v>
-      </c>
-      <c r="B55" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="C55" s="1" t="s">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="11"/>
+      <c r="B56" s="11"/>
+      <c r="C56" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D55" s="1" t="s">
+      <c r="D56" s="1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="10"/>
-      <c r="B56" s="10"/>
-      <c r="C56" s="1" t="s">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="11"/>
+      <c r="B57" s="11"/>
+      <c r="C57" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D56" s="1" t="s">
+      <c r="D57" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="10"/>
-      <c r="B57" s="10"/>
-      <c r="C57" s="1" t="s">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="11"/>
+      <c r="B58" s="11"/>
+      <c r="C58" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D57" s="2" t="s">
+      <c r="D58" s="2" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="10"/>
-      <c r="B58" s="10"/>
-      <c r="C58" s="1" t="s">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="11">
+        <v>18</v>
+      </c>
+      <c r="B59" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="D58" s="2" t="s">
+      <c r="C59" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D59" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="10">
-        <v>18</v>
-      </c>
-      <c r="B59" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="C59" s="1" t="s">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="11"/>
+      <c r="B60" s="11"/>
+      <c r="C60" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D59" s="1" t="s">
+      <c r="D60" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="10"/>
-      <c r="B60" s="10"/>
-      <c r="C60" s="1" t="s">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="11"/>
+      <c r="B61" s="11"/>
+      <c r="C61" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D60" s="1" t="s">
+      <c r="D61" s="2" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="10"/>
-      <c r="B61" s="10"/>
-      <c r="C61" s="1" t="s">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="11"/>
+      <c r="B62" s="11"/>
+      <c r="C62" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D61" s="2" t="s">
+      <c r="D62" s="2" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="10"/>
-      <c r="B62" s="10"/>
-      <c r="C62" s="1" t="s">
+    <row r="63" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A63" s="11">
+        <v>19</v>
+      </c>
+      <c r="B63" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="C63" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D63" s="1" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="63" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A63" s="10">
-        <v>19</v>
-      </c>
-      <c r="B63" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="C63" s="1" t="s">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="11"/>
+      <c r="B64" s="11"/>
+      <c r="C64" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D63" s="1" t="s">
+      <c r="D64" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="10"/>
-      <c r="B64" s="10"/>
-      <c r="C64" s="1" t="s">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="11"/>
+      <c r="B65" s="11"/>
+      <c r="C65" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D64" s="1" t="s">
+      <c r="D65" s="2" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="10"/>
-      <c r="B65" s="10"/>
-      <c r="C65" s="1" t="s">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="11"/>
+      <c r="B66" s="11"/>
+      <c r="C66" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D65" s="2" t="s">
+      <c r="D66" s="2" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="10"/>
-      <c r="B66" s="10"/>
-      <c r="C66" s="1" t="s">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="11">
+        <v>20</v>
+      </c>
+      <c r="B67" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="D66" s="2" t="s">
+      <c r="C67" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="10">
-        <v>20</v>
-      </c>
-      <c r="B67" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="C67" s="1" t="s">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="11"/>
+      <c r="B68" s="11"/>
+      <c r="C68" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D67" s="1" t="s">
+      <c r="D68" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="10"/>
-      <c r="B68" s="10"/>
-      <c r="C68" s="1" t="s">
+    <row r="69" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A69" s="11"/>
+      <c r="B69" s="11"/>
+      <c r="C69" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D68" s="1" t="s">
+      <c r="D69" s="2" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A69" s="10"/>
-      <c r="B69" s="10"/>
-      <c r="C69" s="1" t="s">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="11"/>
+      <c r="B70" s="11"/>
+      <c r="C70" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D69" s="2" t="s">
+      <c r="D70" s="2" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="10"/>
-      <c r="B70" s="10"/>
-      <c r="C70" s="1" t="s">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="11">
+        <v>21</v>
+      </c>
+      <c r="B71" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="D70" s="2" t="s">
+      <c r="C71" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D71" s="1" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="10">
-        <v>21</v>
-      </c>
-      <c r="B71" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="C71" s="1" t="s">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="11"/>
+      <c r="B72" s="11"/>
+      <c r="C72" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D71" s="1" t="s">
+      <c r="D72" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="10"/>
-      <c r="B72" s="10"/>
-      <c r="C72" s="1" t="s">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="11"/>
+      <c r="B73" s="11"/>
+      <c r="C73" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D72" s="1" t="s">
+      <c r="D73" s="2" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="10"/>
-      <c r="B73" s="10"/>
-      <c r="C73" s="1" t="s">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="11"/>
+      <c r="B74" s="11"/>
+      <c r="C74" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D73" s="2" t="s">
+      <c r="D74" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="10"/>
-      <c r="B74" s="10"/>
-      <c r="C74" s="1" t="s">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="11">
+        <v>22</v>
+      </c>
+      <c r="B75" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D74" s="2" t="s">
+      <c r="C75" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D75" s="1" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="10">
-        <v>22</v>
-      </c>
-      <c r="B75" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="C75" s="1" t="s">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="11"/>
+      <c r="B76" s="11"/>
+      <c r="C76" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D75" s="1" t="s">
+      <c r="D76" s="1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="10"/>
-      <c r="B76" s="10"/>
-      <c r="C76" s="1" t="s">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="11"/>
+      <c r="B77" s="11"/>
+      <c r="C77" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D76" s="1" t="s">
+      <c r="D77" s="2" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="10"/>
-      <c r="B77" s="10"/>
-      <c r="C77" s="1" t="s">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="11"/>
+      <c r="B78" s="11"/>
+      <c r="C78" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D77" s="2" t="s">
+      <c r="D78" s="2" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="10"/>
-      <c r="B78" s="10"/>
-      <c r="C78" s="1" t="s">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="11"/>
+      <c r="B79" s="11"/>
+      <c r="C79" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D78" s="2" t="s">
+      <c r="D79" s="2" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="10"/>
-      <c r="B79" s="10"/>
-      <c r="C79" s="1" t="s">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="11">
+        <v>23</v>
+      </c>
+      <c r="B80" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="D79" s="2" t="s">
+      <c r="C80" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D80" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="10">
-        <v>23</v>
-      </c>
-      <c r="B80" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="C80" s="1" t="s">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="11"/>
+      <c r="B81" s="11"/>
+      <c r="C81" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D80" s="1" t="s">
+      <c r="D81" s="1" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="10"/>
-      <c r="B81" s="10"/>
-      <c r="C81" s="1" t="s">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" s="11"/>
+      <c r="B82" s="11"/>
+      <c r="C82" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D81" s="1" t="s">
+      <c r="D82" s="1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="10"/>
-      <c r="B82" s="10"/>
-      <c r="C82" s="1" t="s">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="11">
+        <v>24</v>
+      </c>
+      <c r="B83" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="D82" s="1" t="s">
+      <c r="C83" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D83" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="10">
-        <v>24</v>
-      </c>
-      <c r="B83" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="C83" s="1" t="s">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="11"/>
+      <c r="B84" s="11"/>
+      <c r="C84" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D83" s="1" t="s">
+      <c r="D84" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="10"/>
-      <c r="B84" s="10"/>
-      <c r="C84" s="1" t="s">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="11"/>
+      <c r="B85" s="11"/>
+      <c r="C85" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D84" s="1" t="s">
+      <c r="D85" s="1" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="10"/>
-      <c r="B85" s="10"/>
-      <c r="C85" s="1" t="s">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="11">
+        <v>25</v>
+      </c>
+      <c r="B86" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="D85" s="1" t="s">
+      <c r="C86" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D86" s="1" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="10">
-        <v>25</v>
-      </c>
-      <c r="B86" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="C86" s="1" t="s">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="11"/>
+      <c r="B87" s="11"/>
+      <c r="C87" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D86" s="1" t="s">
+      <c r="D87" s="1" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="10"/>
-      <c r="B87" s="10"/>
-      <c r="C87" s="1" t="s">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="11"/>
+      <c r="B88" s="11"/>
+      <c r="C88" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D87" s="1" t="s">
+      <c r="D88" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="10"/>
-      <c r="B88" s="10"/>
-      <c r="C88" s="1" t="s">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="11"/>
+      <c r="B89" s="11"/>
+      <c r="C89" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D88" s="1" t="s">
+      <c r="D89" s="1" t="s">
         <v>186</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="10"/>
-      <c r="B89" s="10"/>
-      <c r="C89" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D89" s="1" t="s">
-        <v>187</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="B10:B14"/>
-    <mergeCell ref="A15:A21"/>
-    <mergeCell ref="B15:B21"/>
+    <mergeCell ref="B83:B85"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="A83:A85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="B71:B74"/>
+    <mergeCell ref="A71:A74"/>
+    <mergeCell ref="B75:B79"/>
+    <mergeCell ref="A75:A79"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="B80:B82"/>
+    <mergeCell ref="B59:B62"/>
+    <mergeCell ref="A59:A62"/>
+    <mergeCell ref="B63:B66"/>
+    <mergeCell ref="A63:A66"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="A67:A70"/>
+    <mergeCell ref="B46:B54"/>
+    <mergeCell ref="A46:A54"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="B40:B45"/>
+    <mergeCell ref="A40:A45"/>
     <mergeCell ref="B35:B39"/>
     <mergeCell ref="A35:A39"/>
     <mergeCell ref="B7:B9"/>
@@ -2043,33 +2052,18 @@
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="A26:A27"/>
     <mergeCell ref="A10:A14"/>
-    <mergeCell ref="B46:B54"/>
-    <mergeCell ref="A46:A54"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="B40:B45"/>
-    <mergeCell ref="A40:A45"/>
-    <mergeCell ref="B59:B62"/>
-    <mergeCell ref="A59:A62"/>
-    <mergeCell ref="B63:B66"/>
-    <mergeCell ref="A63:A66"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="A67:A70"/>
-    <mergeCell ref="B83:B85"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="A83:A85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="B71:B74"/>
-    <mergeCell ref="A71:A74"/>
-    <mergeCell ref="B75:B79"/>
-    <mergeCell ref="A75:A79"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="B80:B82"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="B10:B14"/>
+    <mergeCell ref="A15:A21"/>
+    <mergeCell ref="B15:B21"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D2 C18:D18 B3:D6 C46 A55:C55 C47:C48 C52:C54 A59:C59 C57:C58 A63:C63 C61:C62 A67:C67 C65:C66 A71:C71 C69:C70 A75:C75 C73:C74 A80:C80 C77:C79 A83:C83 C82 A86:C86 C85 C89 A7:C7 A8:C8 A9:C9 A10:C10 A11:C11 A12:C12 A13:C13 A14:C14 A30:D30 C19 C20 C21 A22:C22 A23:C23 A24:C24 A25:C25 A26:C26 A27:C27 A28:C28 A29:C29 A35:D39 A31:C31 A32:C32 A34:C34 A45:C45 A40:C40 A41:C41 A42:C42 A43:C43 A44:C44 C50 C51 C49 C56 C60 C64 C68 C72 C76 C81 C84 C87 C88" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D2 C18:D18 B3:D6 C46 A55:C55 C47:C48 C52:C54 A59:C59 C57:C58 A63:C63 C61:C62 A67:C67 C65:C66 A71:C71 C69:C70 A75:C75 C73:C74 A80:C80 C77:C79 A83:C83 C82 A86:C86 C85 C89 A7:C7 A8:C8 A9:C9 A10:C10 A11:C11 A12:C12 A13:C13 A14:C14 A30:D30 C19 C21 A22:C22 A23:C23 A24:C24 A25:C25 A26:C26 A27:C27 A28:C28 A29:C29 A35:D39 A31:C31 A32:C32 A34:C34 A45:C45 A40:C40 A41:C41 A42:C42 A43:C43 A44:C44 C50 C51 C49 C56 C60 C64 C68 C72 C76 C81 C84 C87 C88" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
EM-3.4 - Criação da rotina para finalizar compra
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98314F05-207A-426E-9DEC-D7F926ABC9DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F78772F-E9A4-46D6-998A-7977D53EC67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="197">
   <si>
     <t>US</t>
   </si>
@@ -613,6 +613,9 @@
   </si>
   <si>
     <t>Criar rotina para finalização da compra</t>
+  </si>
+  <si>
+    <t>ajustar: RoupasController</t>
   </si>
 </sst>
 </file>
@@ -634,7 +637,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -644,6 +647,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -660,7 +669,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -693,6 +702,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1052,10 +1070,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="10">
+      <c r="A2" s="13">
         <v>1</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="13" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1064,8 +1082,8 @@
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="10"/>
-      <c r="B3" s="10"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
       <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1074,8 +1092,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="10"/>
-      <c r="B4" s="10"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1084,8 +1102,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
       <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1094,8 +1112,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1104,10 +1122,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="11">
+      <c r="A7" s="12">
         <v>2</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="12" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -1118,8 +1136,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="11"/>
-      <c r="B8" s="11"/>
+      <c r="A8" s="12"/>
+      <c r="B8" s="12"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1131,8 +1149,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="11"/>
-      <c r="B9" s="11"/>
+      <c r="A9" s="12"/>
+      <c r="B9" s="12"/>
       <c r="C9" s="6" t="s">
         <v>15</v>
       </c>
@@ -1142,10 +1160,10 @@
       <c r="E9" s="7"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="11">
+      <c r="A10" s="12">
         <v>3</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="12" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1156,8 +1174,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
+      <c r="A11" s="12"/>
+      <c r="B11" s="12"/>
       <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1166,8 +1184,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
+      <c r="A12" s="12"/>
+      <c r="B12" s="12"/>
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
@@ -1176,18 +1194,21 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="7" t="s">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="14" t="s">
         <v>66</v>
       </c>
+      <c r="E13" s="11" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
+      <c r="A14" s="12"/>
+      <c r="B14" s="12"/>
       <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
@@ -1196,10 +1217,10 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11">
+      <c r="A15" s="12">
         <v>4</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="12" t="s">
         <v>25</v>
       </c>
       <c r="C15" s="8" t="s">
@@ -1210,8 +1231,8 @@
       </c>
     </row>
     <row r="16" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
+      <c r="A16" s="12"/>
+      <c r="B16" s="12"/>
       <c r="C16" s="8" t="s">
         <v>191</v>
       </c>
@@ -1220,8 +1241,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
+      <c r="A17" s="12"/>
+      <c r="B17" s="12"/>
       <c r="C17" s="8" t="s">
         <v>194</v>
       </c>
@@ -1230,8 +1251,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="12"/>
       <c r="C18" s="9" t="s">
         <v>26</v>
       </c>
@@ -1240,8 +1261,8 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
       <c r="C19" s="9" t="s">
         <v>28</v>
       </c>
@@ -1250,18 +1271,18 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="1" t="s">
+      <c r="A20" s="12"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="10" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="11"/>
-      <c r="B21" s="11"/>
+      <c r="A21" s="12"/>
+      <c r="B21" s="12"/>
       <c r="C21" s="1" t="s">
         <v>29</v>
       </c>
@@ -1270,10 +1291,10 @@
       </c>
     </row>
     <row r="22" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="11">
+      <c r="A22" s="12">
         <v>5</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="12" t="s">
         <v>30</v>
       </c>
       <c r="C22" s="1" t="s">
@@ -1284,8 +1305,8 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="11"/>
-      <c r="B23" s="11"/>
+      <c r="A23" s="12"/>
+      <c r="B23" s="12"/>
       <c r="C23" s="1" t="s">
         <v>32</v>
       </c>
@@ -1294,10 +1315,10 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="11">
+      <c r="A24" s="12">
         <v>6</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="12" t="s">
         <v>33</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -1308,8 +1329,8 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="11"/>
-      <c r="B25" s="11"/>
+      <c r="A25" s="12"/>
+      <c r="B25" s="12"/>
       <c r="C25" s="1" t="s">
         <v>35</v>
       </c>
@@ -1318,10 +1339,10 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="11">
+      <c r="A26" s="12">
         <v>7</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="12" t="s">
         <v>36</v>
       </c>
       <c r="C26" s="1" t="s">
@@ -1332,8 +1353,8 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11"/>
+      <c r="A27" s="12"/>
+      <c r="B27" s="12"/>
       <c r="C27" s="1" t="s">
         <v>38</v>
       </c>
@@ -1398,10 +1419,10 @@
       </c>
     </row>
     <row r="32" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="11">
+      <c r="A32" s="12">
         <v>12</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C32" s="1" t="s">
@@ -1412,8 +1433,8 @@
       </c>
     </row>
     <row r="33" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="11"/>
-      <c r="B33" s="11"/>
+      <c r="A33" s="12"/>
+      <c r="B33" s="12"/>
       <c r="C33" s="2" t="s">
         <v>134</v>
       </c>
@@ -1436,48 +1457,48 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="10">
+      <c r="A35" s="13">
         <v>14</v>
       </c>
-      <c r="B35" s="10" t="s">
+      <c r="B35" s="13" t="s">
         <v>52</v>
       </c>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
+      <c r="A36" s="13"/>
+      <c r="B36" s="13"/>
       <c r="C36" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D36" s="3"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="10"/>
-      <c r="B37" s="10"/>
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
       <c r="C37" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D37" s="3"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="10"/>
-      <c r="B38" s="10"/>
+      <c r="A38" s="13"/>
+      <c r="B38" s="13"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="10"/>
-      <c r="B39" s="10"/>
+      <c r="A39" s="13"/>
+      <c r="B39" s="13"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="11">
+      <c r="A40" s="12">
         <v>15</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="12" t="s">
         <v>55</v>
       </c>
       <c r="C40" s="1" t="s">
@@ -1488,8 +1509,8 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="11"/>
-      <c r="B41" s="11"/>
+      <c r="A41" s="12"/>
+      <c r="B41" s="12"/>
       <c r="C41" s="1" t="s">
         <v>57</v>
       </c>
@@ -1498,8 +1519,8 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="11"/>
-      <c r="B42" s="11"/>
+      <c r="A42" s="12"/>
+      <c r="B42" s="12"/>
       <c r="C42" s="1" t="s">
         <v>58</v>
       </c>
@@ -1508,8 +1529,8 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="11"/>
-      <c r="B43" s="11"/>
+      <c r="A43" s="12"/>
+      <c r="B43" s="12"/>
       <c r="C43" s="1" t="s">
         <v>59</v>
       </c>
@@ -1518,8 +1539,8 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="11"/>
-      <c r="B44" s="11"/>
+      <c r="A44" s="12"/>
+      <c r="B44" s="12"/>
       <c r="C44" s="1" t="s">
         <v>60</v>
       </c>
@@ -1528,8 +1549,8 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="11"/>
-      <c r="B45" s="11"/>
+      <c r="A45" s="12"/>
+      <c r="B45" s="12"/>
       <c r="C45" s="1" t="s">
         <v>61</v>
       </c>
@@ -1538,10 +1559,10 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="11">
+      <c r="A46" s="12">
         <v>16</v>
       </c>
-      <c r="B46" s="11" t="s">
+      <c r="B46" s="12" t="s">
         <v>73</v>
       </c>
       <c r="C46" s="1" t="s">
@@ -1552,8 +1573,8 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="11"/>
-      <c r="B47" s="11"/>
+      <c r="A47" s="12"/>
+      <c r="B47" s="12"/>
       <c r="C47" s="1" t="s">
         <v>63</v>
       </c>
@@ -1562,8 +1583,8 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="11"/>
-      <c r="B48" s="11"/>
+      <c r="A48" s="12"/>
+      <c r="B48" s="12"/>
       <c r="C48" s="1" t="s">
         <v>64</v>
       </c>
@@ -1572,8 +1593,8 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="11"/>
-      <c r="B49" s="11"/>
+      <c r="A49" s="12"/>
+      <c r="B49" s="12"/>
       <c r="C49" s="1" t="s">
         <v>65</v>
       </c>
@@ -1582,8 +1603,8 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="11"/>
-      <c r="B50" s="11"/>
+      <c r="A50" s="12"/>
+      <c r="B50" s="12"/>
       <c r="C50" s="1" t="s">
         <v>68</v>
       </c>
@@ -1592,8 +1613,8 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="11"/>
-      <c r="B51" s="11"/>
+      <c r="A51" s="12"/>
+      <c r="B51" s="12"/>
       <c r="C51" s="1" t="s">
         <v>72</v>
       </c>
@@ -1602,8 +1623,8 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="11"/>
-      <c r="B52" s="11"/>
+      <c r="A52" s="12"/>
+      <c r="B52" s="12"/>
       <c r="C52" s="1" t="s">
         <v>74</v>
       </c>
@@ -1612,8 +1633,8 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="11"/>
-      <c r="B53" s="11"/>
+      <c r="A53" s="12"/>
+      <c r="B53" s="12"/>
       <c r="C53" s="1" t="s">
         <v>75</v>
       </c>
@@ -1622,8 +1643,8 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="11"/>
-      <c r="B54" s="11"/>
+      <c r="A54" s="12"/>
+      <c r="B54" s="12"/>
       <c r="C54" s="1" t="s">
         <v>76</v>
       </c>
@@ -1632,10 +1653,10 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="11">
+      <c r="A55" s="12">
         <v>17</v>
       </c>
-      <c r="B55" s="11" t="s">
+      <c r="B55" s="12" t="s">
         <v>77</v>
       </c>
       <c r="C55" s="1" t="s">
@@ -1646,8 +1667,8 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="11"/>
-      <c r="B56" s="11"/>
+      <c r="A56" s="12"/>
+      <c r="B56" s="12"/>
       <c r="C56" s="1" t="s">
         <v>79</v>
       </c>
@@ -1656,8 +1677,8 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="11"/>
-      <c r="B57" s="11"/>
+      <c r="A57" s="12"/>
+      <c r="B57" s="12"/>
       <c r="C57" s="1" t="s">
         <v>80</v>
       </c>
@@ -1666,8 +1687,8 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="11"/>
-      <c r="B58" s="11"/>
+      <c r="A58" s="12"/>
+      <c r="B58" s="12"/>
       <c r="C58" s="1" t="s">
         <v>81</v>
       </c>
@@ -1676,10 +1697,10 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="11">
+      <c r="A59" s="12">
         <v>18</v>
       </c>
-      <c r="B59" s="11" t="s">
+      <c r="B59" s="12" t="s">
         <v>82</v>
       </c>
       <c r="C59" s="1" t="s">
@@ -1690,8 +1711,8 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="11"/>
-      <c r="B60" s="11"/>
+      <c r="A60" s="12"/>
+      <c r="B60" s="12"/>
       <c r="C60" s="1" t="s">
         <v>84</v>
       </c>
@@ -1700,8 +1721,8 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="11"/>
-      <c r="B61" s="11"/>
+      <c r="A61" s="12"/>
+      <c r="B61" s="12"/>
       <c r="C61" s="1" t="s">
         <v>85</v>
       </c>
@@ -1710,8 +1731,8 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="11"/>
-      <c r="B62" s="11"/>
+      <c r="A62" s="12"/>
+      <c r="B62" s="12"/>
       <c r="C62" s="1" t="s">
         <v>86</v>
       </c>
@@ -1720,10 +1741,10 @@
       </c>
     </row>
     <row r="63" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A63" s="11">
+      <c r="A63" s="12">
         <v>19</v>
       </c>
-      <c r="B63" s="11" t="s">
+      <c r="B63" s="12" t="s">
         <v>87</v>
       </c>
       <c r="C63" s="1" t="s">
@@ -1734,8 +1755,8 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="11"/>
-      <c r="B64" s="11"/>
+      <c r="A64" s="12"/>
+      <c r="B64" s="12"/>
       <c r="C64" s="1" t="s">
         <v>89</v>
       </c>
@@ -1744,8 +1765,8 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="11"/>
-      <c r="B65" s="11"/>
+      <c r="A65" s="12"/>
+      <c r="B65" s="12"/>
       <c r="C65" s="1" t="s">
         <v>90</v>
       </c>
@@ -1754,8 +1775,8 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="11"/>
-      <c r="B66" s="11"/>
+      <c r="A66" s="12"/>
+      <c r="B66" s="12"/>
       <c r="C66" s="1" t="s">
         <v>91</v>
       </c>
@@ -1764,10 +1785,10 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="11">
+      <c r="A67" s="12">
         <v>20</v>
       </c>
-      <c r="B67" s="11" t="s">
+      <c r="B67" s="12" t="s">
         <v>92</v>
       </c>
       <c r="C67" s="1" t="s">
@@ -1778,8 +1799,8 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="11"/>
-      <c r="B68" s="11"/>
+      <c r="A68" s="12"/>
+      <c r="B68" s="12"/>
       <c r="C68" s="1" t="s">
         <v>94</v>
       </c>
@@ -1788,8 +1809,8 @@
       </c>
     </row>
     <row r="69" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A69" s="11"/>
-      <c r="B69" s="11"/>
+      <c r="A69" s="12"/>
+      <c r="B69" s="12"/>
       <c r="C69" s="1" t="s">
         <v>95</v>
       </c>
@@ -1798,8 +1819,8 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="11"/>
-      <c r="B70" s="11"/>
+      <c r="A70" s="12"/>
+      <c r="B70" s="12"/>
       <c r="C70" s="1" t="s">
         <v>96</v>
       </c>
@@ -1808,10 +1829,10 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="11">
+      <c r="A71" s="12">
         <v>21</v>
       </c>
-      <c r="B71" s="11" t="s">
+      <c r="B71" s="12" t="s">
         <v>97</v>
       </c>
       <c r="C71" s="1" t="s">
@@ -1822,8 +1843,8 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="11"/>
-      <c r="B72" s="11"/>
+      <c r="A72" s="12"/>
+      <c r="B72" s="12"/>
       <c r="C72" s="1" t="s">
         <v>99</v>
       </c>
@@ -1832,8 +1853,8 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="11"/>
-      <c r="B73" s="11"/>
+      <c r="A73" s="12"/>
+      <c r="B73" s="12"/>
       <c r="C73" s="1" t="s">
         <v>100</v>
       </c>
@@ -1842,8 +1863,8 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="11"/>
-      <c r="B74" s="11"/>
+      <c r="A74" s="12"/>
+      <c r="B74" s="12"/>
       <c r="C74" s="1" t="s">
         <v>101</v>
       </c>
@@ -1852,10 +1873,10 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="11">
+      <c r="A75" s="12">
         <v>22</v>
       </c>
-      <c r="B75" s="11" t="s">
+      <c r="B75" s="12" t="s">
         <v>102</v>
       </c>
       <c r="C75" s="1" t="s">
@@ -1866,8 +1887,8 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="11"/>
-      <c r="B76" s="11"/>
+      <c r="A76" s="12"/>
+      <c r="B76" s="12"/>
       <c r="C76" s="1" t="s">
         <v>104</v>
       </c>
@@ -1876,8 +1897,8 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="11"/>
-      <c r="B77" s="11"/>
+      <c r="A77" s="12"/>
+      <c r="B77" s="12"/>
       <c r="C77" s="1" t="s">
         <v>105</v>
       </c>
@@ -1886,8 +1907,8 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="11"/>
-      <c r="B78" s="11"/>
+      <c r="A78" s="12"/>
+      <c r="B78" s="12"/>
       <c r="C78" s="1" t="s">
         <v>106</v>
       </c>
@@ -1896,8 +1917,8 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="11"/>
-      <c r="B79" s="11"/>
+      <c r="A79" s="12"/>
+      <c r="B79" s="12"/>
       <c r="C79" s="1" t="s">
         <v>107</v>
       </c>
@@ -1906,10 +1927,10 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="11">
+      <c r="A80" s="12">
         <v>23</v>
       </c>
-      <c r="B80" s="11" t="s">
+      <c r="B80" s="12" t="s">
         <v>108</v>
       </c>
       <c r="C80" s="1" t="s">
@@ -1920,8 +1941,8 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="11"/>
-      <c r="B81" s="11"/>
+      <c r="A81" s="12"/>
+      <c r="B81" s="12"/>
       <c r="C81" s="1" t="s">
         <v>110</v>
       </c>
@@ -1930,8 +1951,8 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="11"/>
-      <c r="B82" s="11"/>
+      <c r="A82" s="12"/>
+      <c r="B82" s="12"/>
       <c r="C82" s="1" t="s">
         <v>111</v>
       </c>
@@ -1940,10 +1961,10 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="11">
+      <c r="A83" s="12">
         <v>24</v>
       </c>
-      <c r="B83" s="11" t="s">
+      <c r="B83" s="12" t="s">
         <v>112</v>
       </c>
       <c r="C83" s="1" t="s">
@@ -1954,8 +1975,8 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="11"/>
-      <c r="B84" s="11"/>
+      <c r="A84" s="12"/>
+      <c r="B84" s="12"/>
       <c r="C84" s="1" t="s">
         <v>114</v>
       </c>
@@ -1964,8 +1985,8 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="11"/>
-      <c r="B85" s="11"/>
+      <c r="A85" s="12"/>
+      <c r="B85" s="12"/>
       <c r="C85" s="1" t="s">
         <v>115</v>
       </c>
@@ -1974,10 +1995,10 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="11">
+      <c r="A86" s="12">
         <v>25</v>
       </c>
-      <c r="B86" s="11" t="s">
+      <c r="B86" s="12" t="s">
         <v>116</v>
       </c>
       <c r="C86" s="1" t="s">
@@ -1988,8 +2009,8 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="11"/>
-      <c r="B87" s="11"/>
+      <c r="A87" s="12"/>
+      <c r="B87" s="12"/>
       <c r="C87" s="1" t="s">
         <v>118</v>
       </c>
@@ -1998,8 +2019,8 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="11"/>
-      <c r="B88" s="11"/>
+      <c r="A88" s="12"/>
+      <c r="B88" s="12"/>
       <c r="C88" s="1" t="s">
         <v>119</v>
       </c>
@@ -2008,8 +2029,8 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="11"/>
-      <c r="B89" s="11"/>
+      <c r="A89" s="12"/>
+      <c r="B89" s="12"/>
       <c r="C89" s="1" t="s">
         <v>120</v>
       </c>
@@ -2019,28 +2040,13 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="B83:B85"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="A83:A85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="B71:B74"/>
-    <mergeCell ref="A71:A74"/>
-    <mergeCell ref="B75:B79"/>
-    <mergeCell ref="A75:A79"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="B80:B82"/>
-    <mergeCell ref="B59:B62"/>
-    <mergeCell ref="A59:A62"/>
-    <mergeCell ref="B63:B66"/>
-    <mergeCell ref="A63:A66"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="A67:A70"/>
-    <mergeCell ref="B46:B54"/>
-    <mergeCell ref="A46:A54"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="B40:B45"/>
-    <mergeCell ref="A40:A45"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="B10:B14"/>
+    <mergeCell ref="A15:A21"/>
+    <mergeCell ref="B15:B21"/>
     <mergeCell ref="B35:B39"/>
     <mergeCell ref="A35:A39"/>
     <mergeCell ref="B7:B9"/>
@@ -2052,13 +2058,28 @@
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="A26:A27"/>
     <mergeCell ref="A10:A14"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="B10:B14"/>
-    <mergeCell ref="A15:A21"/>
-    <mergeCell ref="B15:B21"/>
+    <mergeCell ref="B46:B54"/>
+    <mergeCell ref="A46:A54"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="B40:B45"/>
+    <mergeCell ref="A40:A45"/>
+    <mergeCell ref="B59:B62"/>
+    <mergeCell ref="A59:A62"/>
+    <mergeCell ref="B63:B66"/>
+    <mergeCell ref="A63:A66"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="A67:A70"/>
+    <mergeCell ref="B83:B85"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="A83:A85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="B71:B74"/>
+    <mergeCell ref="A71:A74"/>
+    <mergeCell ref="B75:B79"/>
+    <mergeCell ref="A75:A79"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="B80:B82"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
EM-3.4 - Implementado lógica para retornar produtos tela principal
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F78772F-E9A4-46D6-998A-7977D53EC67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43A50730-4028-4352-9275-695BE38C669F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-900" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
   <si>
     <t>US</t>
   </si>
@@ -613,9 +613,6 @@
   </si>
   <si>
     <t>Criar rotina para finalização da compra</t>
-  </si>
-  <si>
-    <t>ajustar: RoupasController</t>
   </si>
 </sst>
 </file>
@@ -637,7 +634,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -647,12 +644,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -704,13 +695,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1122,10 +1113,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
+      <c r="A7" s="14">
         <v>2</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="14" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -1136,8 +1127,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1149,8 +1140,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
+      <c r="A9" s="14"/>
+      <c r="B9" s="14"/>
       <c r="C9" s="6" t="s">
         <v>15</v>
       </c>
@@ -1160,10 +1151,10 @@
       <c r="E9" s="7"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
+      <c r="A10" s="14">
         <v>3</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="14" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1174,8 +1165,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
+      <c r="A11" s="14"/>
+      <c r="B11" s="14"/>
       <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1184,8 +1175,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12"/>
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
@@ -1194,21 +1185,19 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="14" t="s">
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="E13" s="11" t="s">
-        <v>196</v>
-      </c>
+      <c r="E13" s="11"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12"/>
+      <c r="A14" s="14"/>
+      <c r="B14" s="14"/>
       <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
@@ -1217,10 +1206,10 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12">
+      <c r="A15" s="14">
         <v>4</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="14" t="s">
         <v>25</v>
       </c>
       <c r="C15" s="8" t="s">
@@ -1231,8 +1220,8 @@
       </c>
     </row>
     <row r="16" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12"/>
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
       <c r="C16" s="8" t="s">
         <v>191</v>
       </c>
@@ -1241,8 +1230,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
+      <c r="A17" s="14"/>
+      <c r="B17" s="14"/>
       <c r="C17" s="8" t="s">
         <v>194</v>
       </c>
@@ -1251,8 +1240,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
       <c r="C18" s="9" t="s">
         <v>26</v>
       </c>
@@ -1261,8 +1250,8 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
+      <c r="A19" s="14"/>
+      <c r="B19" s="14"/>
       <c r="C19" s="9" t="s">
         <v>28</v>
       </c>
@@ -1271,8 +1260,8 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
+      <c r="A20" s="14"/>
+      <c r="B20" s="14"/>
       <c r="C20" s="10" t="s">
         <v>195</v>
       </c>
@@ -1281,8 +1270,8 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
+      <c r="A21" s="14"/>
+      <c r="B21" s="14"/>
       <c r="C21" s="1" t="s">
         <v>29</v>
       </c>
@@ -1291,10 +1280,10 @@
       </c>
     </row>
     <row r="22" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="12">
+      <c r="A22" s="14">
         <v>5</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="14" t="s">
         <v>30</v>
       </c>
       <c r="C22" s="1" t="s">
@@ -1305,8 +1294,8 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12"/>
+      <c r="A23" s="14"/>
+      <c r="B23" s="14"/>
       <c r="C23" s="1" t="s">
         <v>32</v>
       </c>
@@ -1315,10 +1304,10 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="12">
+      <c r="A24" s="14">
         <v>6</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="14" t="s">
         <v>33</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -1329,8 +1318,8 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
+      <c r="A25" s="14"/>
+      <c r="B25" s="14"/>
       <c r="C25" s="1" t="s">
         <v>35</v>
       </c>
@@ -1339,10 +1328,10 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="12">
+      <c r="A26" s="14">
         <v>7</v>
       </c>
-      <c r="B26" s="12" t="s">
+      <c r="B26" s="14" t="s">
         <v>36</v>
       </c>
       <c r="C26" s="1" t="s">
@@ -1353,8 +1342,8 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12"/>
+      <c r="A27" s="14"/>
+      <c r="B27" s="14"/>
       <c r="C27" s="1" t="s">
         <v>38</v>
       </c>
@@ -1419,10 +1408,10 @@
       </c>
     </row>
     <row r="32" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="12">
+      <c r="A32" s="14">
         <v>12</v>
       </c>
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="14" t="s">
         <v>48</v>
       </c>
       <c r="C32" s="1" t="s">
@@ -1433,8 +1422,8 @@
       </c>
     </row>
     <row r="33" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="12"/>
-      <c r="B33" s="12"/>
+      <c r="A33" s="14"/>
+      <c r="B33" s="14"/>
       <c r="C33" s="2" t="s">
         <v>134</v>
       </c>
@@ -1495,10 +1484,10 @@
       <c r="D39" s="3"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="12">
+      <c r="A40" s="14">
         <v>15</v>
       </c>
-      <c r="B40" s="12" t="s">
+      <c r="B40" s="14" t="s">
         <v>55</v>
       </c>
       <c r="C40" s="1" t="s">
@@ -1509,8 +1498,8 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="12"/>
-      <c r="B41" s="12"/>
+      <c r="A41" s="14"/>
+      <c r="B41" s="14"/>
       <c r="C41" s="1" t="s">
         <v>57</v>
       </c>
@@ -1519,8 +1508,8 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="12"/>
-      <c r="B42" s="12"/>
+      <c r="A42" s="14"/>
+      <c r="B42" s="14"/>
       <c r="C42" s="1" t="s">
         <v>58</v>
       </c>
@@ -1529,8 +1518,8 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="12"/>
-      <c r="B43" s="12"/>
+      <c r="A43" s="14"/>
+      <c r="B43" s="14"/>
       <c r="C43" s="1" t="s">
         <v>59</v>
       </c>
@@ -1539,8 +1528,8 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="12"/>
-      <c r="B44" s="12"/>
+      <c r="A44" s="14"/>
+      <c r="B44" s="14"/>
       <c r="C44" s="1" t="s">
         <v>60</v>
       </c>
@@ -1549,8 +1538,8 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="12"/>
-      <c r="B45" s="12"/>
+      <c r="A45" s="14"/>
+      <c r="B45" s="14"/>
       <c r="C45" s="1" t="s">
         <v>61</v>
       </c>
@@ -1559,10 +1548,10 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="12">
+      <c r="A46" s="14">
         <v>16</v>
       </c>
-      <c r="B46" s="12" t="s">
+      <c r="B46" s="14" t="s">
         <v>73</v>
       </c>
       <c r="C46" s="1" t="s">
@@ -1573,8 +1562,8 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="12"/>
-      <c r="B47" s="12"/>
+      <c r="A47" s="14"/>
+      <c r="B47" s="14"/>
       <c r="C47" s="1" t="s">
         <v>63</v>
       </c>
@@ -1583,8 +1572,8 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="12"/>
-      <c r="B48" s="12"/>
+      <c r="A48" s="14"/>
+      <c r="B48" s="14"/>
       <c r="C48" s="1" t="s">
         <v>64</v>
       </c>
@@ -1593,8 +1582,8 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="12"/>
-      <c r="B49" s="12"/>
+      <c r="A49" s="14"/>
+      <c r="B49" s="14"/>
       <c r="C49" s="1" t="s">
         <v>65</v>
       </c>
@@ -1603,8 +1592,8 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="12"/>
-      <c r="B50" s="12"/>
+      <c r="A50" s="14"/>
+      <c r="B50" s="14"/>
       <c r="C50" s="1" t="s">
         <v>68</v>
       </c>
@@ -1613,8 +1602,8 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="12"/>
-      <c r="B51" s="12"/>
+      <c r="A51" s="14"/>
+      <c r="B51" s="14"/>
       <c r="C51" s="1" t="s">
         <v>72</v>
       </c>
@@ -1623,8 +1612,8 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="12"/>
-      <c r="B52" s="12"/>
+      <c r="A52" s="14"/>
+      <c r="B52" s="14"/>
       <c r="C52" s="1" t="s">
         <v>74</v>
       </c>
@@ -1633,8 +1622,8 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="12"/>
-      <c r="B53" s="12"/>
+      <c r="A53" s="14"/>
+      <c r="B53" s="14"/>
       <c r="C53" s="1" t="s">
         <v>75</v>
       </c>
@@ -1643,8 +1632,8 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="12"/>
-      <c r="B54" s="12"/>
+      <c r="A54" s="14"/>
+      <c r="B54" s="14"/>
       <c r="C54" s="1" t="s">
         <v>76</v>
       </c>
@@ -1653,10 +1642,10 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="12">
+      <c r="A55" s="14">
         <v>17</v>
       </c>
-      <c r="B55" s="12" t="s">
+      <c r="B55" s="14" t="s">
         <v>77</v>
       </c>
       <c r="C55" s="1" t="s">
@@ -1667,8 +1656,8 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="12"/>
-      <c r="B56" s="12"/>
+      <c r="A56" s="14"/>
+      <c r="B56" s="14"/>
       <c r="C56" s="1" t="s">
         <v>79</v>
       </c>
@@ -1677,8 +1666,8 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="12"/>
-      <c r="B57" s="12"/>
+      <c r="A57" s="14"/>
+      <c r="B57" s="14"/>
       <c r="C57" s="1" t="s">
         <v>80</v>
       </c>
@@ -1687,8 +1676,8 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="12"/>
-      <c r="B58" s="12"/>
+      <c r="A58" s="14"/>
+      <c r="B58" s="14"/>
       <c r="C58" s="1" t="s">
         <v>81</v>
       </c>
@@ -1697,10 +1686,10 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="12">
+      <c r="A59" s="14">
         <v>18</v>
       </c>
-      <c r="B59" s="12" t="s">
+      <c r="B59" s="14" t="s">
         <v>82</v>
       </c>
       <c r="C59" s="1" t="s">
@@ -1711,8 +1700,8 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="12"/>
-      <c r="B60" s="12"/>
+      <c r="A60" s="14"/>
+      <c r="B60" s="14"/>
       <c r="C60" s="1" t="s">
         <v>84</v>
       </c>
@@ -1721,8 +1710,8 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="12"/>
-      <c r="B61" s="12"/>
+      <c r="A61" s="14"/>
+      <c r="B61" s="14"/>
       <c r="C61" s="1" t="s">
         <v>85</v>
       </c>
@@ -1731,8 +1720,8 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="12"/>
-      <c r="B62" s="12"/>
+      <c r="A62" s="14"/>
+      <c r="B62" s="14"/>
       <c r="C62" s="1" t="s">
         <v>86</v>
       </c>
@@ -1741,10 +1730,10 @@
       </c>
     </row>
     <row r="63" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A63" s="12">
+      <c r="A63" s="14">
         <v>19</v>
       </c>
-      <c r="B63" s="12" t="s">
+      <c r="B63" s="14" t="s">
         <v>87</v>
       </c>
       <c r="C63" s="1" t="s">
@@ -1755,8 +1744,8 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="12"/>
-      <c r="B64" s="12"/>
+      <c r="A64" s="14"/>
+      <c r="B64" s="14"/>
       <c r="C64" s="1" t="s">
         <v>89</v>
       </c>
@@ -1765,8 +1754,8 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="12"/>
-      <c r="B65" s="12"/>
+      <c r="A65" s="14"/>
+      <c r="B65" s="14"/>
       <c r="C65" s="1" t="s">
         <v>90</v>
       </c>
@@ -1775,8 +1764,8 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="12"/>
-      <c r="B66" s="12"/>
+      <c r="A66" s="14"/>
+      <c r="B66" s="14"/>
       <c r="C66" s="1" t="s">
         <v>91</v>
       </c>
@@ -1785,10 +1774,10 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="12">
+      <c r="A67" s="14">
         <v>20</v>
       </c>
-      <c r="B67" s="12" t="s">
+      <c r="B67" s="14" t="s">
         <v>92</v>
       </c>
       <c r="C67" s="1" t="s">
@@ -1799,8 +1788,8 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="12"/>
-      <c r="B68" s="12"/>
+      <c r="A68" s="14"/>
+      <c r="B68" s="14"/>
       <c r="C68" s="1" t="s">
         <v>94</v>
       </c>
@@ -1809,8 +1798,8 @@
       </c>
     </row>
     <row r="69" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A69" s="12"/>
-      <c r="B69" s="12"/>
+      <c r="A69" s="14"/>
+      <c r="B69" s="14"/>
       <c r="C69" s="1" t="s">
         <v>95</v>
       </c>
@@ -1819,8 +1808,8 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="12"/>
-      <c r="B70" s="12"/>
+      <c r="A70" s="14"/>
+      <c r="B70" s="14"/>
       <c r="C70" s="1" t="s">
         <v>96</v>
       </c>
@@ -1829,10 +1818,10 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="12">
+      <c r="A71" s="14">
         <v>21</v>
       </c>
-      <c r="B71" s="12" t="s">
+      <c r="B71" s="14" t="s">
         <v>97</v>
       </c>
       <c r="C71" s="1" t="s">
@@ -1843,8 +1832,8 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="12"/>
-      <c r="B72" s="12"/>
+      <c r="A72" s="14"/>
+      <c r="B72" s="14"/>
       <c r="C72" s="1" t="s">
         <v>99</v>
       </c>
@@ -1853,8 +1842,8 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="12"/>
-      <c r="B73" s="12"/>
+      <c r="A73" s="14"/>
+      <c r="B73" s="14"/>
       <c r="C73" s="1" t="s">
         <v>100</v>
       </c>
@@ -1863,8 +1852,8 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="12"/>
-      <c r="B74" s="12"/>
+      <c r="A74" s="14"/>
+      <c r="B74" s="14"/>
       <c r="C74" s="1" t="s">
         <v>101</v>
       </c>
@@ -1873,10 +1862,10 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="12">
+      <c r="A75" s="14">
         <v>22</v>
       </c>
-      <c r="B75" s="12" t="s">
+      <c r="B75" s="14" t="s">
         <v>102</v>
       </c>
       <c r="C75" s="1" t="s">
@@ -1887,8 +1876,8 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="12"/>
-      <c r="B76" s="12"/>
+      <c r="A76" s="14"/>
+      <c r="B76" s="14"/>
       <c r="C76" s="1" t="s">
         <v>104</v>
       </c>
@@ -1897,8 +1886,8 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="12"/>
-      <c r="B77" s="12"/>
+      <c r="A77" s="14"/>
+      <c r="B77" s="14"/>
       <c r="C77" s="1" t="s">
         <v>105</v>
       </c>
@@ -1907,8 +1896,8 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="12"/>
-      <c r="B78" s="12"/>
+      <c r="A78" s="14"/>
+      <c r="B78" s="14"/>
       <c r="C78" s="1" t="s">
         <v>106</v>
       </c>
@@ -1917,8 +1906,8 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="12"/>
-      <c r="B79" s="12"/>
+      <c r="A79" s="14"/>
+      <c r="B79" s="14"/>
       <c r="C79" s="1" t="s">
         <v>107</v>
       </c>
@@ -1927,10 +1916,10 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="12">
+      <c r="A80" s="14">
         <v>23</v>
       </c>
-      <c r="B80" s="12" t="s">
+      <c r="B80" s="14" t="s">
         <v>108</v>
       </c>
       <c r="C80" s="1" t="s">
@@ -1941,8 +1930,8 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="12"/>
-      <c r="B81" s="12"/>
+      <c r="A81" s="14"/>
+      <c r="B81" s="14"/>
       <c r="C81" s="1" t="s">
         <v>110</v>
       </c>
@@ -1951,8 +1940,8 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="12"/>
-      <c r="B82" s="12"/>
+      <c r="A82" s="14"/>
+      <c r="B82" s="14"/>
       <c r="C82" s="1" t="s">
         <v>111</v>
       </c>
@@ -1961,10 +1950,10 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="12">
+      <c r="A83" s="14">
         <v>24</v>
       </c>
-      <c r="B83" s="12" t="s">
+      <c r="B83" s="14" t="s">
         <v>112</v>
       </c>
       <c r="C83" s="1" t="s">
@@ -1975,8 +1964,8 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="12"/>
-      <c r="B84" s="12"/>
+      <c r="A84" s="14"/>
+      <c r="B84" s="14"/>
       <c r="C84" s="1" t="s">
         <v>114</v>
       </c>
@@ -1985,8 +1974,8 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="12"/>
-      <c r="B85" s="12"/>
+      <c r="A85" s="14"/>
+      <c r="B85" s="14"/>
       <c r="C85" s="1" t="s">
         <v>115</v>
       </c>
@@ -1995,10 +1984,10 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="12">
+      <c r="A86" s="14">
         <v>25</v>
       </c>
-      <c r="B86" s="12" t="s">
+      <c r="B86" s="14" t="s">
         <v>116</v>
       </c>
       <c r="C86" s="1" t="s">
@@ -2009,8 +1998,8 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="12"/>
-      <c r="B87" s="12"/>
+      <c r="A87" s="14"/>
+      <c r="B87" s="14"/>
       <c r="C87" s="1" t="s">
         <v>118</v>
       </c>
@@ -2019,8 +2008,8 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="12"/>
-      <c r="B88" s="12"/>
+      <c r="A88" s="14"/>
+      <c r="B88" s="14"/>
       <c r="C88" s="1" t="s">
         <v>119</v>
       </c>
@@ -2029,8 +2018,8 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="12"/>
-      <c r="B89" s="12"/>
+      <c r="A89" s="14"/>
+      <c r="B89" s="14"/>
       <c r="C89" s="1" t="s">
         <v>120</v>
       </c>
@@ -2040,13 +2029,28 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="B10:B14"/>
-    <mergeCell ref="A15:A21"/>
-    <mergeCell ref="B15:B21"/>
+    <mergeCell ref="B83:B85"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="A83:A85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="B71:B74"/>
+    <mergeCell ref="A71:A74"/>
+    <mergeCell ref="B75:B79"/>
+    <mergeCell ref="A75:A79"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="B80:B82"/>
+    <mergeCell ref="B59:B62"/>
+    <mergeCell ref="A59:A62"/>
+    <mergeCell ref="B63:B66"/>
+    <mergeCell ref="A63:A66"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="A67:A70"/>
+    <mergeCell ref="B46:B54"/>
+    <mergeCell ref="A46:A54"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="B40:B45"/>
+    <mergeCell ref="A40:A45"/>
     <mergeCell ref="B35:B39"/>
     <mergeCell ref="A35:A39"/>
     <mergeCell ref="B7:B9"/>
@@ -2058,28 +2062,13 @@
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="A26:A27"/>
     <mergeCell ref="A10:A14"/>
-    <mergeCell ref="B46:B54"/>
-    <mergeCell ref="A46:A54"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="B40:B45"/>
-    <mergeCell ref="A40:A45"/>
-    <mergeCell ref="B59:B62"/>
-    <mergeCell ref="A59:A62"/>
-    <mergeCell ref="B63:B66"/>
-    <mergeCell ref="A63:A66"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="A67:A70"/>
-    <mergeCell ref="B83:B85"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="A83:A85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="B71:B74"/>
-    <mergeCell ref="A71:A74"/>
-    <mergeCell ref="B75:B79"/>
-    <mergeCell ref="A75:A79"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="B80:B82"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="B10:B14"/>
+    <mergeCell ref="A15:A21"/>
+    <mergeCell ref="B15:B21"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
EM-3.6 - Tela de detalhes dos produtos
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43A50730-4028-4352-9275-695BE38C669F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0AD7849-8EEE-4E32-ADC7-7E81C7F70221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-900" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="198">
   <si>
     <t>US</t>
   </si>
@@ -613,6 +613,12 @@
   </si>
   <si>
     <t>Criar rotina para finalização da compra</t>
+  </si>
+  <si>
+    <t>3.6</t>
+  </si>
+  <si>
+    <t>Criar tela para o usuário visualizar individualmente os produtos</t>
   </si>
 </sst>
 </file>
@@ -634,7 +640,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -644,6 +650,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -660,7 +672,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -702,6 +714,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1038,7 +1059,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
@@ -1061,10 +1082,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="13">
+      <c r="A2" s="16">
         <v>1</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="16" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1073,8 +1094,8 @@
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
+      <c r="A3" s="16"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1083,8 +1104,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="16"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1093,8 +1114,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="13"/>
-      <c r="B5" s="13"/>
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1103,8 +1124,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="13"/>
-      <c r="B6" s="13"/>
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1113,10 +1134,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="14">
+      <c r="A7" s="15">
         <v>2</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="15" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -1127,8 +1148,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="14"/>
-      <c r="B8" s="14"/>
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1140,8 +1161,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
-      <c r="B9" s="14"/>
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
       <c r="C9" s="6" t="s">
         <v>15</v>
       </c>
@@ -1150,11 +1171,11 @@
       </c>
       <c r="E9" s="7"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="14">
+    <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="15">
         <v>3</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="15" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1165,8 +1186,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="14"/>
-      <c r="B11" s="14"/>
+      <c r="A11" s="15"/>
+      <c r="B11" s="15"/>
       <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1175,8 +1196,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
-      <c r="B12" s="14"/>
+      <c r="A12" s="15"/>
+      <c r="B12" s="15"/>
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
@@ -1185,8 +1206,8 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="14"/>
-      <c r="B13" s="14"/>
+      <c r="A13" s="15"/>
+      <c r="B13" s="15"/>
       <c r="C13" s="12" t="s">
         <v>21</v>
       </c>
@@ -1196,8 +1217,8 @@
       <c r="E13" s="11"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="14"/>
-      <c r="B14" s="14"/>
+      <c r="A14" s="15"/>
+      <c r="B14" s="15"/>
       <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
@@ -1205,875 +1226,885 @@
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="14">
+    <row r="15" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="15"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="15">
         <v>4</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B16" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C16" s="8" t="s">
         <v>189</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D16" s="8" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="14"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="8" t="s">
+    <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D17" s="8" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="14"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="8" t="s">
+    <row r="18" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="15"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D18" s="8" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="9" t="s">
+    <row r="19" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D19" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="14"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="9" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D20" s="9" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="14"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="10" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="15"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D21" s="10" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="14"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="1" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="15"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D22" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="14">
+    <row r="23" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="15">
         <v>5</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B23" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C23" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D23" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="14"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="1" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="15"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D24" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="14">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="15">
         <v>6</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B25" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C25" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="14"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="1" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="15"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D26" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="14">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="15">
         <v>7</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B27" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="14"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="1" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="15"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D28" s="1" t="s">
         <v>129</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
-        <v>8</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>45</v>
+        <v>131</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
+        <v>10</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
         <v>11</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B32" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C32" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D32" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="14">
+    <row r="33" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="15">
         <v>12</v>
       </c>
-      <c r="B32" s="14" t="s">
+      <c r="B33" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C33" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="33" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="14"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="2" t="s">
+    <row r="34" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="15"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D34" s="2" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
+    <row r="35" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
         <v>13</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B35" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C35" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="D35" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="13">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="16">
         <v>14</v>
       </c>
-      <c r="B35" s="13" t="s">
+      <c r="B36" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="13"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="16"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D36" s="3"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="13"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="3" t="s">
+      <c r="D37" s="3"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="16"/>
+      <c r="B38" s="16"/>
+      <c r="C38" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D37" s="3"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="13"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="3"/>
       <c r="D38" s="3"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="13"/>
-      <c r="B39" s="13"/>
+      <c r="A39" s="16"/>
+      <c r="B39" s="16"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="14">
+      <c r="A40" s="16"/>
+      <c r="B40" s="16"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="15">
         <v>15</v>
       </c>
-      <c r="B40" s="14" t="s">
+      <c r="B41" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C41" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D41" s="13" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="14"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="1" t="s">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="15"/>
+      <c r="B42" s="15"/>
+      <c r="C42" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="D42" s="13" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="14"/>
-      <c r="B42" s="14"/>
-      <c r="C42" s="1" t="s">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="15"/>
+      <c r="B43" s="15"/>
+      <c r="C43" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="D43" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="14"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="1" t="s">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="15"/>
+      <c r="B44" s="15"/>
+      <c r="C44" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="D44" s="13" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="14"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="1" t="s">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="15"/>
+      <c r="B45" s="15"/>
+      <c r="C45" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="D45" s="13" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="14"/>
-      <c r="B45" s="14"/>
-      <c r="C45" s="1" t="s">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="15"/>
+      <c r="B46" s="15"/>
+      <c r="C46" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="D46" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="14">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="15">
         <v>16</v>
       </c>
-      <c r="B46" s="14" t="s">
+      <c r="B47" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C47" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="D47" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="14"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="1" t="s">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="15"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D47" s="1" t="s">
+      <c r="D48" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="14"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="1" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="15"/>
+      <c r="B49" s="15"/>
+      <c r="C49" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="D49" s="2" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="14"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="1" t="s">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="15"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D49" s="2" t="s">
+      <c r="D50" s="2" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="14"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="1" t="s">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="15"/>
+      <c r="B51" s="15"/>
+      <c r="C51" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D50" s="2" t="s">
+      <c r="D51" s="2" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="14"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="1" t="s">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="15"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D51" s="2" t="s">
+      <c r="D52" s="2" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="14"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="1" t="s">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="15"/>
+      <c r="B53" s="15"/>
+      <c r="C53" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D52" s="2" t="s">
+      <c r="D53" s="2" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="14"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="1" t="s">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="15"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D53" s="2" t="s">
+      <c r="D54" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="14"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="1" t="s">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="15"/>
+      <c r="B55" s="15"/>
+      <c r="C55" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D54" s="2" t="s">
+      <c r="D55" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="14">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="15">
         <v>17</v>
       </c>
-      <c r="B55" s="14" t="s">
+      <c r="B56" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="C55" s="1" t="s">
+      <c r="C56" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D55" s="1" t="s">
+      <c r="D56" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="14"/>
-      <c r="B56" s="14"/>
-      <c r="C56" s="1" t="s">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="15"/>
+      <c r="B57" s="15"/>
+      <c r="C57" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D56" s="1" t="s">
+      <c r="D57" s="1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="14"/>
-      <c r="B57" s="14"/>
-      <c r="C57" s="1" t="s">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="15"/>
+      <c r="B58" s="15"/>
+      <c r="C58" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D57" s="2" t="s">
+      <c r="D58" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="14"/>
-      <c r="B58" s="14"/>
-      <c r="C58" s="1" t="s">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="15"/>
+      <c r="B59" s="15"/>
+      <c r="C59" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D58" s="2" t="s">
+      <c r="D59" s="2" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="14">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="15">
         <v>18</v>
       </c>
-      <c r="B59" s="14" t="s">
+      <c r="B60" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="C60" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D59" s="1" t="s">
+      <c r="D60" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="14"/>
-      <c r="B60" s="14"/>
-      <c r="C60" s="1" t="s">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="15"/>
+      <c r="B61" s="15"/>
+      <c r="C61" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D60" s="1" t="s">
+      <c r="D61" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="14"/>
-      <c r="B61" s="14"/>
-      <c r="C61" s="1" t="s">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="15"/>
+      <c r="B62" s="15"/>
+      <c r="C62" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D61" s="2" t="s">
+      <c r="D62" s="2" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="14"/>
-      <c r="B62" s="14"/>
-      <c r="C62" s="1" t="s">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="15"/>
+      <c r="B63" s="15"/>
+      <c r="C63" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="D63" s="2" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="63" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A63" s="14">
+    <row r="64" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A64" s="15">
         <v>19</v>
       </c>
-      <c r="B63" s="14" t="s">
+      <c r="B64" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="C63" s="1" t="s">
+      <c r="C64" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D63" s="1" t="s">
+      <c r="D64" s="1" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="14"/>
-      <c r="B64" s="14"/>
-      <c r="C64" s="1" t="s">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="15"/>
+      <c r="B65" s="15"/>
+      <c r="C65" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D64" s="1" t="s">
+      <c r="D65" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="14"/>
-      <c r="B65" s="14"/>
-      <c r="C65" s="1" t="s">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="15"/>
+      <c r="B66" s="15"/>
+      <c r="C66" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D65" s="2" t="s">
+      <c r="D66" s="2" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="14"/>
-      <c r="B66" s="14"/>
-      <c r="C66" s="1" t="s">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="15"/>
+      <c r="B67" s="15"/>
+      <c r="C67" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D66" s="2" t="s">
+      <c r="D67" s="2" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="14">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="15">
         <v>20</v>
       </c>
-      <c r="B67" s="14" t="s">
+      <c r="B68" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="C67" s="1" t="s">
+      <c r="C68" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="D67" s="1" t="s">
+      <c r="D68" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="14"/>
-      <c r="B68" s="14"/>
-      <c r="C68" s="1" t="s">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="15"/>
+      <c r="B69" s="15"/>
+      <c r="C69" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D68" s="1" t="s">
+      <c r="D69" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A69" s="14"/>
-      <c r="B69" s="14"/>
-      <c r="C69" s="1" t="s">
+    <row r="70" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A70" s="15"/>
+      <c r="B70" s="15"/>
+      <c r="C70" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D69" s="2" t="s">
+      <c r="D70" s="2" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="14"/>
-      <c r="B70" s="14"/>
-      <c r="C70" s="1" t="s">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="15"/>
+      <c r="B71" s="15"/>
+      <c r="C71" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D70" s="2" t="s">
+      <c r="D71" s="2" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="14">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="15">
         <v>21</v>
       </c>
-      <c r="B71" s="14" t="s">
+      <c r="B72" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="C71" s="1" t="s">
+      <c r="C72" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D71" s="1" t="s">
+      <c r="D72" s="1" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="14"/>
-      <c r="B72" s="14"/>
-      <c r="C72" s="1" t="s">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="15"/>
+      <c r="B73" s="15"/>
+      <c r="C73" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D72" s="1" t="s">
+      <c r="D73" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="14"/>
-      <c r="B73" s="14"/>
-      <c r="C73" s="1" t="s">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="15"/>
+      <c r="B74" s="15"/>
+      <c r="C74" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D73" s="2" t="s">
+      <c r="D74" s="2" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="14"/>
-      <c r="B74" s="14"/>
-      <c r="C74" s="1" t="s">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="15"/>
+      <c r="B75" s="15"/>
+      <c r="C75" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D74" s="2" t="s">
+      <c r="D75" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="14">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="15">
         <v>22</v>
       </c>
-      <c r="B75" s="14" t="s">
+      <c r="B76" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="C75" s="1" t="s">
+      <c r="C76" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D75" s="1" t="s">
+      <c r="D76" s="1" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="14"/>
-      <c r="B76" s="14"/>
-      <c r="C76" s="1" t="s">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="15"/>
+      <c r="B77" s="15"/>
+      <c r="C77" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D76" s="1" t="s">
+      <c r="D77" s="1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="14"/>
-      <c r="B77" s="14"/>
-      <c r="C77" s="1" t="s">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="15"/>
+      <c r="B78" s="15"/>
+      <c r="C78" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D77" s="2" t="s">
+      <c r="D78" s="2" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="14"/>
-      <c r="B78" s="14"/>
-      <c r="C78" s="1" t="s">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="15"/>
+      <c r="B79" s="15"/>
+      <c r="C79" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D78" s="2" t="s">
+      <c r="D79" s="2" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="14"/>
-      <c r="B79" s="14"/>
-      <c r="C79" s="1" t="s">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="15"/>
+      <c r="B80" s="15"/>
+      <c r="C80" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D79" s="2" t="s">
+      <c r="D80" s="2" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="14">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="15">
         <v>23</v>
       </c>
-      <c r="B80" s="14" t="s">
+      <c r="B81" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="C80" s="1" t="s">
+      <c r="C81" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D80" s="1" t="s">
+      <c r="D81" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="14"/>
-      <c r="B81" s="14"/>
-      <c r="C81" s="1" t="s">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" s="15"/>
+      <c r="B82" s="15"/>
+      <c r="C82" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D81" s="1" t="s">
+      <c r="D82" s="1" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="14"/>
-      <c r="B82" s="14"/>
-      <c r="C82" s="1" t="s">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="15"/>
+      <c r="B83" s="15"/>
+      <c r="C83" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D82" s="1" t="s">
+      <c r="D83" s="1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="14">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="15">
         <v>24</v>
       </c>
-      <c r="B83" s="14" t="s">
+      <c r="B84" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="C83" s="1" t="s">
+      <c r="C84" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D83" s="1" t="s">
+      <c r="D84" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="14"/>
-      <c r="B84" s="14"/>
-      <c r="C84" s="1" t="s">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="15"/>
+      <c r="B85" s="15"/>
+      <c r="C85" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D84" s="1" t="s">
+      <c r="D85" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="14"/>
-      <c r="B85" s="14"/>
-      <c r="C85" s="1" t="s">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="15"/>
+      <c r="B86" s="15"/>
+      <c r="C86" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D85" s="1" t="s">
+      <c r="D86" s="1" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="14">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="15">
         <v>25</v>
       </c>
-      <c r="B86" s="14" t="s">
+      <c r="B87" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="C86" s="1" t="s">
+      <c r="C87" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D86" s="1" t="s">
+      <c r="D87" s="1" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="14"/>
-      <c r="B87" s="14"/>
-      <c r="C87" s="1" t="s">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="15"/>
+      <c r="B88" s="15"/>
+      <c r="C88" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D87" s="1" t="s">
+      <c r="D88" s="1" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="14"/>
-      <c r="B88" s="14"/>
-      <c r="C88" s="1" t="s">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="15"/>
+      <c r="B89" s="15"/>
+      <c r="C89" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D88" s="1" t="s">
+      <c r="D89" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="14"/>
-      <c r="B89" s="14"/>
-      <c r="C89" s="1" t="s">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" s="15"/>
+      <c r="B90" s="15"/>
+      <c r="C90" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D89" s="1" t="s">
+      <c r="D90" s="1" t="s">
         <v>186</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="B83:B85"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="A83:A85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="B71:B74"/>
-    <mergeCell ref="A71:A74"/>
-    <mergeCell ref="B75:B79"/>
-    <mergeCell ref="A75:A79"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="B80:B82"/>
-    <mergeCell ref="B59:B62"/>
-    <mergeCell ref="A59:A62"/>
-    <mergeCell ref="B63:B66"/>
-    <mergeCell ref="A63:A66"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="A67:A70"/>
-    <mergeCell ref="B46:B54"/>
-    <mergeCell ref="A46:A54"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="B40:B45"/>
-    <mergeCell ref="A40:A45"/>
-    <mergeCell ref="B35:B39"/>
-    <mergeCell ref="A35:A39"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A10:A14"/>
     <mergeCell ref="B2:B6"/>
     <mergeCell ref="A2:A6"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="B10:B14"/>
-    <mergeCell ref="A15:A21"/>
-    <mergeCell ref="B15:B21"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A16:A22"/>
+    <mergeCell ref="B16:B22"/>
+    <mergeCell ref="A10:A15"/>
+    <mergeCell ref="B10:B15"/>
+    <mergeCell ref="B36:B40"/>
+    <mergeCell ref="A36:A40"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B47:B55"/>
+    <mergeCell ref="A47:A55"/>
+    <mergeCell ref="B56:B59"/>
+    <mergeCell ref="A56:A59"/>
+    <mergeCell ref="B41:B46"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="B60:B63"/>
+    <mergeCell ref="A60:A63"/>
+    <mergeCell ref="B64:B67"/>
+    <mergeCell ref="A64:A67"/>
+    <mergeCell ref="B68:B71"/>
+    <mergeCell ref="A68:A71"/>
+    <mergeCell ref="B84:B86"/>
+    <mergeCell ref="B87:B90"/>
+    <mergeCell ref="A84:A86"/>
+    <mergeCell ref="A87:A90"/>
+    <mergeCell ref="B72:B75"/>
+    <mergeCell ref="A72:A75"/>
+    <mergeCell ref="B76:B80"/>
+    <mergeCell ref="A76:A80"/>
+    <mergeCell ref="A81:A83"/>
+    <mergeCell ref="B81:B83"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D2 C18:D18 B3:D6 C46 A55:C55 C47:C48 C52:C54 A59:C59 C57:C58 A63:C63 C61:C62 A67:C67 C65:C66 A71:C71 C69:C70 A75:C75 C73:C74 A80:C80 C77:C79 A83:C83 C82 A86:C86 C85 C89 A7:C7 A8:C8 A9:C9 A10:C10 A11:C11 A12:C12 A13:C13 A14:C14 A30:D30 C19 C21 A22:C22 A23:C23 A24:C24 A25:C25 A26:C26 A27:C27 A28:C28 A29:C29 A35:D39 A31:C31 A32:C32 A34:C34 A45:C45 A40:C40 A41:C41 A42:C42 A43:C43 A44:C44 C50 C51 C49 C56 C60 C64 C68 C72 C76 C81 C84 C87 C88" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D2 C19:D19 B3:D6 C47 A56:C56 C48:C49 C53:C55 A60:C60 C58:C59 A64:C64 C62:C63 A68:C68 C66:C67 A72:C72 C70:C71 A76:C76 C74:C75 A81:C81 C78:C80 A84:C84 C83 A87:C87 C86 C90 A7:C7 A8:C8 A9:C9 A10:C10 C11 C12 C13 C14 A31:D31 C20 C22 A23:C23 A24:C24 A25:C25 A26:C26 A27:C27 A28:C28 A29:C29 A30:C30 A36:D40 A32:C32 A33:C33 A35:C35 A46:C46 A41:C41 A42:C42 A43:C43 A44:C44 A45:C45 C51 C52 C50 C57 C61 C65 C69 C73 C77 C82 C85 C88 C89" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
EM-10.1 - Implementado lógica para retornar produtos mais vendidos e produtos novos
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0AD7849-8EEE-4E32-ADC7-7E81C7F70221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47BBBEEF-27F7-4A92-A80D-686D5DE26291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-900" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -640,7 +640,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -650,12 +650,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -716,13 +710,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1134,10 +1128,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="15">
+      <c r="A7" s="17">
         <v>2</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="17" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -1148,8 +1142,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1161,8 +1155,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="15"/>
-      <c r="B9" s="15"/>
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
       <c r="C9" s="6" t="s">
         <v>15</v>
       </c>
@@ -1172,10 +1166,10 @@
       <c r="E9" s="7"/>
     </row>
     <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="15">
+      <c r="A10" s="17">
         <v>3</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="17" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1186,8 +1180,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
       <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1196,8 +1190,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="15"/>
-      <c r="B12" s="15"/>
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
@@ -1206,8 +1200,8 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="15"/>
-      <c r="B13" s="15"/>
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
       <c r="C13" s="12" t="s">
         <v>21</v>
       </c>
@@ -1217,8 +1211,8 @@
       <c r="E13" s="11"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="15"/>
-      <c r="B14" s="15"/>
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
       <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
@@ -1227,20 +1221,20 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="15"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="17" t="s">
+      <c r="A15" s="17"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="15" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="15">
+      <c r="A16" s="17">
         <v>4</v>
       </c>
-      <c r="B16" s="15" t="s">
+      <c r="B16" s="17" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="8" t="s">
@@ -1251,8 +1245,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="15"/>
-      <c r="B17" s="15"/>
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
       <c r="C17" s="8" t="s">
         <v>191</v>
       </c>
@@ -1261,8 +1255,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="15"/>
-      <c r="B18" s="15"/>
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
       <c r="C18" s="8" t="s">
         <v>194</v>
       </c>
@@ -1271,8 +1265,8 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="15"/>
-      <c r="B19" s="15"/>
+      <c r="A19" s="17"/>
+      <c r="B19" s="17"/>
       <c r="C19" s="9" t="s">
         <v>26</v>
       </c>
@@ -1281,8 +1275,8 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="15"/>
-      <c r="B20" s="15"/>
+      <c r="A20" s="17"/>
+      <c r="B20" s="17"/>
       <c r="C20" s="9" t="s">
         <v>28</v>
       </c>
@@ -1291,8 +1285,8 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="15"/>
-      <c r="B21" s="15"/>
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
       <c r="C21" s="10" t="s">
         <v>195</v>
       </c>
@@ -1301,8 +1295,8 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15"/>
+      <c r="A22" s="17"/>
+      <c r="B22" s="17"/>
       <c r="C22" s="1" t="s">
         <v>29</v>
       </c>
@@ -1311,10 +1305,10 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
+      <c r="A23" s="17">
         <v>5</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="B23" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -1325,8 +1319,8 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="15"/>
-      <c r="B24" s="15"/>
+      <c r="A24" s="17"/>
+      <c r="B24" s="17"/>
       <c r="C24" s="1" t="s">
         <v>32</v>
       </c>
@@ -1335,10 +1329,10 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="15">
+      <c r="A25" s="17">
         <v>6</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="17" t="s">
         <v>33</v>
       </c>
       <c r="C25" s="1" t="s">
@@ -1349,8 +1343,8 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="15"/>
-      <c r="B26" s="15"/>
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
       <c r="C26" s="1" t="s">
         <v>35</v>
       </c>
@@ -1359,10 +1353,10 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="15">
+      <c r="A27" s="17">
         <v>7</v>
       </c>
-      <c r="B27" s="15" t="s">
+      <c r="B27" s="17" t="s">
         <v>36</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -1373,8 +1367,8 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
-      <c r="B28" s="15"/>
+      <c r="A28" s="17"/>
+      <c r="B28" s="17"/>
       <c r="C28" s="1" t="s">
         <v>38</v>
       </c>
@@ -1439,10 +1433,10 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="15">
+      <c r="A33" s="17">
         <v>12</v>
       </c>
-      <c r="B33" s="15" t="s">
+      <c r="B33" s="17" t="s">
         <v>48</v>
       </c>
       <c r="C33" s="1" t="s">
@@ -1453,8 +1447,8 @@
       </c>
     </row>
     <row r="34" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="15"/>
-      <c r="B34" s="15"/>
+      <c r="A34" s="17"/>
+      <c r="B34" s="17"/>
       <c r="C34" s="2" t="s">
         <v>134</v>
       </c>
@@ -1515,10 +1509,10 @@
       <c r="D40" s="3"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="15">
+      <c r="A41" s="17">
         <v>15</v>
       </c>
-      <c r="B41" s="15" t="s">
+      <c r="B41" s="17" t="s">
         <v>55</v>
       </c>
       <c r="C41" s="13" t="s">
@@ -1529,8 +1523,8 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="15"/>
-      <c r="B42" s="15"/>
+      <c r="A42" s="17"/>
+      <c r="B42" s="17"/>
       <c r="C42" s="13" t="s">
         <v>57</v>
       </c>
@@ -1539,8 +1533,8 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="15"/>
-      <c r="B43" s="15"/>
+      <c r="A43" s="17"/>
+      <c r="B43" s="17"/>
       <c r="C43" s="1" t="s">
         <v>58</v>
       </c>
@@ -1549,8 +1543,8 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="15"/>
-      <c r="B44" s="15"/>
+      <c r="A44" s="17"/>
+      <c r="B44" s="17"/>
       <c r="C44" s="13" t="s">
         <v>59</v>
       </c>
@@ -1559,8 +1553,8 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="15"/>
-      <c r="B45" s="15"/>
+      <c r="A45" s="17"/>
+      <c r="B45" s="17"/>
       <c r="C45" s="13" t="s">
         <v>60</v>
       </c>
@@ -1569,8 +1563,8 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="15"/>
-      <c r="B46" s="15"/>
+      <c r="A46" s="17"/>
+      <c r="B46" s="17"/>
       <c r="C46" s="1" t="s">
         <v>61</v>
       </c>
@@ -1579,10 +1573,10 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="15">
+      <c r="A47" s="17">
         <v>16</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="B47" s="17" t="s">
         <v>73</v>
       </c>
       <c r="C47" s="1" t="s">
@@ -1593,8 +1587,8 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="15"/>
-      <c r="B48" s="15"/>
+      <c r="A48" s="17"/>
+      <c r="B48" s="17"/>
       <c r="C48" s="1" t="s">
         <v>63</v>
       </c>
@@ -1603,8 +1597,8 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="15"/>
-      <c r="B49" s="15"/>
+      <c r="A49" s="17"/>
+      <c r="B49" s="17"/>
       <c r="C49" s="1" t="s">
         <v>64</v>
       </c>
@@ -1613,8 +1607,8 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="15"/>
-      <c r="B50" s="15"/>
+      <c r="A50" s="17"/>
+      <c r="B50" s="17"/>
       <c r="C50" s="1" t="s">
         <v>65</v>
       </c>
@@ -1623,8 +1617,8 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="15"/>
-      <c r="B51" s="15"/>
+      <c r="A51" s="17"/>
+      <c r="B51" s="17"/>
       <c r="C51" s="1" t="s">
         <v>68</v>
       </c>
@@ -1633,8 +1627,8 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="15"/>
-      <c r="B52" s="15"/>
+      <c r="A52" s="17"/>
+      <c r="B52" s="17"/>
       <c r="C52" s="1" t="s">
         <v>72</v>
       </c>
@@ -1643,8 +1637,8 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="15"/>
-      <c r="B53" s="15"/>
+      <c r="A53" s="17"/>
+      <c r="B53" s="17"/>
       <c r="C53" s="1" t="s">
         <v>74</v>
       </c>
@@ -1653,8 +1647,8 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="15"/>
-      <c r="B54" s="15"/>
+      <c r="A54" s="17"/>
+      <c r="B54" s="17"/>
       <c r="C54" s="1" t="s">
         <v>75</v>
       </c>
@@ -1663,8 +1657,8 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="15"/>
-      <c r="B55" s="15"/>
+      <c r="A55" s="17"/>
+      <c r="B55" s="17"/>
       <c r="C55" s="1" t="s">
         <v>76</v>
       </c>
@@ -1673,10 +1667,10 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="15">
+      <c r="A56" s="17">
         <v>17</v>
       </c>
-      <c r="B56" s="15" t="s">
+      <c r="B56" s="17" t="s">
         <v>77</v>
       </c>
       <c r="C56" s="1" t="s">
@@ -1687,8 +1681,8 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="15"/>
-      <c r="B57" s="15"/>
+      <c r="A57" s="17"/>
+      <c r="B57" s="17"/>
       <c r="C57" s="1" t="s">
         <v>79</v>
       </c>
@@ -1697,8 +1691,8 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="15"/>
-      <c r="B58" s="15"/>
+      <c r="A58" s="17"/>
+      <c r="B58" s="17"/>
       <c r="C58" s="1" t="s">
         <v>80</v>
       </c>
@@ -1707,8 +1701,8 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="15"/>
-      <c r="B59" s="15"/>
+      <c r="A59" s="17"/>
+      <c r="B59" s="17"/>
       <c r="C59" s="1" t="s">
         <v>81</v>
       </c>
@@ -1717,10 +1711,10 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="15">
+      <c r="A60" s="17">
         <v>18</v>
       </c>
-      <c r="B60" s="15" t="s">
+      <c r="B60" s="17" t="s">
         <v>82</v>
       </c>
       <c r="C60" s="1" t="s">
@@ -1731,8 +1725,8 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="15"/>
-      <c r="B61" s="15"/>
+      <c r="A61" s="17"/>
+      <c r="B61" s="17"/>
       <c r="C61" s="1" t="s">
         <v>84</v>
       </c>
@@ -1741,8 +1735,8 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="15"/>
-      <c r="B62" s="15"/>
+      <c r="A62" s="17"/>
+      <c r="B62" s="17"/>
       <c r="C62" s="1" t="s">
         <v>85</v>
       </c>
@@ -1751,8 +1745,8 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="15"/>
-      <c r="B63" s="15"/>
+      <c r="A63" s="17"/>
+      <c r="B63" s="17"/>
       <c r="C63" s="1" t="s">
         <v>86</v>
       </c>
@@ -1761,10 +1755,10 @@
       </c>
     </row>
     <row r="64" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A64" s="15">
+      <c r="A64" s="17">
         <v>19</v>
       </c>
-      <c r="B64" s="15" t="s">
+      <c r="B64" s="17" t="s">
         <v>87</v>
       </c>
       <c r="C64" s="1" t="s">
@@ -1775,8 +1769,8 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="15"/>
-      <c r="B65" s="15"/>
+      <c r="A65" s="17"/>
+      <c r="B65" s="17"/>
       <c r="C65" s="1" t="s">
         <v>89</v>
       </c>
@@ -1785,8 +1779,8 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="15"/>
-      <c r="B66" s="15"/>
+      <c r="A66" s="17"/>
+      <c r="B66" s="17"/>
       <c r="C66" s="1" t="s">
         <v>90</v>
       </c>
@@ -1795,8 +1789,8 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="15"/>
-      <c r="B67" s="15"/>
+      <c r="A67" s="17"/>
+      <c r="B67" s="17"/>
       <c r="C67" s="1" t="s">
         <v>91</v>
       </c>
@@ -1805,10 +1799,10 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="15">
+      <c r="A68" s="17">
         <v>20</v>
       </c>
-      <c r="B68" s="15" t="s">
+      <c r="B68" s="17" t="s">
         <v>92</v>
       </c>
       <c r="C68" s="1" t="s">
@@ -1819,8 +1813,8 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="15"/>
-      <c r="B69" s="15"/>
+      <c r="A69" s="17"/>
+      <c r="B69" s="17"/>
       <c r="C69" s="1" t="s">
         <v>94</v>
       </c>
@@ -1829,8 +1823,8 @@
       </c>
     </row>
     <row r="70" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A70" s="15"/>
-      <c r="B70" s="15"/>
+      <c r="A70" s="17"/>
+      <c r="B70" s="17"/>
       <c r="C70" s="1" t="s">
         <v>95</v>
       </c>
@@ -1839,8 +1833,8 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="15"/>
-      <c r="B71" s="15"/>
+      <c r="A71" s="17"/>
+      <c r="B71" s="17"/>
       <c r="C71" s="1" t="s">
         <v>96</v>
       </c>
@@ -1849,10 +1843,10 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="15">
+      <c r="A72" s="17">
         <v>21</v>
       </c>
-      <c r="B72" s="15" t="s">
+      <c r="B72" s="17" t="s">
         <v>97</v>
       </c>
       <c r="C72" s="1" t="s">
@@ -1863,8 +1857,8 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="15"/>
-      <c r="B73" s="15"/>
+      <c r="A73" s="17"/>
+      <c r="B73" s="17"/>
       <c r="C73" s="1" t="s">
         <v>99</v>
       </c>
@@ -1873,8 +1867,8 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="15"/>
-      <c r="B74" s="15"/>
+      <c r="A74" s="17"/>
+      <c r="B74" s="17"/>
       <c r="C74" s="1" t="s">
         <v>100</v>
       </c>
@@ -1883,8 +1877,8 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="15"/>
-      <c r="B75" s="15"/>
+      <c r="A75" s="17"/>
+      <c r="B75" s="17"/>
       <c r="C75" s="1" t="s">
         <v>101</v>
       </c>
@@ -1893,10 +1887,10 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="15">
+      <c r="A76" s="17">
         <v>22</v>
       </c>
-      <c r="B76" s="15" t="s">
+      <c r="B76" s="17" t="s">
         <v>102</v>
       </c>
       <c r="C76" s="1" t="s">
@@ -1907,8 +1901,8 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="15"/>
-      <c r="B77" s="15"/>
+      <c r="A77" s="17"/>
+      <c r="B77" s="17"/>
       <c r="C77" s="1" t="s">
         <v>104</v>
       </c>
@@ -1917,8 +1911,8 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="15"/>
-      <c r="B78" s="15"/>
+      <c r="A78" s="17"/>
+      <c r="B78" s="17"/>
       <c r="C78" s="1" t="s">
         <v>105</v>
       </c>
@@ -1927,8 +1921,8 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="15"/>
-      <c r="B79" s="15"/>
+      <c r="A79" s="17"/>
+      <c r="B79" s="17"/>
       <c r="C79" s="1" t="s">
         <v>106</v>
       </c>
@@ -1937,8 +1931,8 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="15"/>
-      <c r="B80" s="15"/>
+      <c r="A80" s="17"/>
+      <c r="B80" s="17"/>
       <c r="C80" s="1" t="s">
         <v>107</v>
       </c>
@@ -1947,10 +1941,10 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="15">
+      <c r="A81" s="17">
         <v>23</v>
       </c>
-      <c r="B81" s="15" t="s">
+      <c r="B81" s="17" t="s">
         <v>108</v>
       </c>
       <c r="C81" s="1" t="s">
@@ -1961,8 +1955,8 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="15"/>
-      <c r="B82" s="15"/>
+      <c r="A82" s="17"/>
+      <c r="B82" s="17"/>
       <c r="C82" s="1" t="s">
         <v>110</v>
       </c>
@@ -1971,8 +1965,8 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="15"/>
-      <c r="B83" s="15"/>
+      <c r="A83" s="17"/>
+      <c r="B83" s="17"/>
       <c r="C83" s="1" t="s">
         <v>111</v>
       </c>
@@ -1981,10 +1975,10 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="15">
+      <c r="A84" s="17">
         <v>24</v>
       </c>
-      <c r="B84" s="15" t="s">
+      <c r="B84" s="17" t="s">
         <v>112</v>
       </c>
       <c r="C84" s="1" t="s">
@@ -1995,8 +1989,8 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="15"/>
-      <c r="B85" s="15"/>
+      <c r="A85" s="17"/>
+      <c r="B85" s="17"/>
       <c r="C85" s="1" t="s">
         <v>114</v>
       </c>
@@ -2005,8 +1999,8 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="15"/>
-      <c r="B86" s="15"/>
+      <c r="A86" s="17"/>
+      <c r="B86" s="17"/>
       <c r="C86" s="1" t="s">
         <v>115</v>
       </c>
@@ -2015,10 +2009,10 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="15">
+      <c r="A87" s="17">
         <v>25</v>
       </c>
-      <c r="B87" s="15" t="s">
+      <c r="B87" s="17" t="s">
         <v>116</v>
       </c>
       <c r="C87" s="1" t="s">
@@ -2029,8 +2023,8 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="15"/>
-      <c r="B88" s="15"/>
+      <c r="A88" s="17"/>
+      <c r="B88" s="17"/>
       <c r="C88" s="1" t="s">
         <v>118</v>
       </c>
@@ -2039,8 +2033,8 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="15"/>
-      <c r="B89" s="15"/>
+      <c r="A89" s="17"/>
+      <c r="B89" s="17"/>
       <c r="C89" s="1" t="s">
         <v>119</v>
       </c>
@@ -2049,8 +2043,8 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="15"/>
-      <c r="B90" s="15"/>
+      <c r="A90" s="17"/>
+      <c r="B90" s="17"/>
       <c r="C90" s="1" t="s">
         <v>120</v>
       </c>
@@ -2060,14 +2054,28 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A16:A22"/>
-    <mergeCell ref="B16:B22"/>
-    <mergeCell ref="A10:A15"/>
-    <mergeCell ref="B10:B15"/>
+    <mergeCell ref="B84:B86"/>
+    <mergeCell ref="B87:B90"/>
+    <mergeCell ref="A84:A86"/>
+    <mergeCell ref="A87:A90"/>
+    <mergeCell ref="B72:B75"/>
+    <mergeCell ref="A72:A75"/>
+    <mergeCell ref="B76:B80"/>
+    <mergeCell ref="A76:A80"/>
+    <mergeCell ref="A81:A83"/>
+    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="B60:B63"/>
+    <mergeCell ref="A60:A63"/>
+    <mergeCell ref="B64:B67"/>
+    <mergeCell ref="A64:A67"/>
+    <mergeCell ref="B68:B71"/>
+    <mergeCell ref="A68:A71"/>
+    <mergeCell ref="B47:B55"/>
+    <mergeCell ref="A47:A55"/>
+    <mergeCell ref="B56:B59"/>
+    <mergeCell ref="A56:A59"/>
+    <mergeCell ref="B41:B46"/>
+    <mergeCell ref="A41:A46"/>
     <mergeCell ref="B36:B40"/>
     <mergeCell ref="A36:A40"/>
     <mergeCell ref="B7:B9"/>
@@ -2078,28 +2086,14 @@
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B47:B55"/>
-    <mergeCell ref="A47:A55"/>
-    <mergeCell ref="B56:B59"/>
-    <mergeCell ref="A56:A59"/>
-    <mergeCell ref="B41:B46"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="B60:B63"/>
-    <mergeCell ref="A60:A63"/>
-    <mergeCell ref="B64:B67"/>
-    <mergeCell ref="A64:A67"/>
-    <mergeCell ref="B68:B71"/>
-    <mergeCell ref="A68:A71"/>
-    <mergeCell ref="B84:B86"/>
-    <mergeCell ref="B87:B90"/>
-    <mergeCell ref="A84:A86"/>
-    <mergeCell ref="A87:A90"/>
-    <mergeCell ref="B72:B75"/>
-    <mergeCell ref="A72:A75"/>
-    <mergeCell ref="B76:B80"/>
-    <mergeCell ref="A76:A80"/>
-    <mergeCell ref="A81:A83"/>
-    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A16:A22"/>
+    <mergeCell ref="B16:B22"/>
+    <mergeCell ref="A10:A15"/>
+    <mergeCell ref="B10:B15"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
EM-12.1,12.2 - Rotina para visualizar as compras
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47BBBEEF-27F7-4A92-A80D-686D5DE26291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED3F14C-3E97-4F24-9C0B-06BB3B6D7915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-900" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -640,7 +640,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -650,6 +650,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -666,7 +672,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -710,13 +716,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1076,10 +1088,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="16">
+      <c r="A2" s="18">
         <v>1</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1088,8 +1100,8 @@
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
       <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1098,8 +1110,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1108,8 +1120,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16"/>
+      <c r="A5" s="18"/>
+      <c r="B5" s="18"/>
       <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1118,8 +1130,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
-      <c r="B6" s="16"/>
+      <c r="A6" s="18"/>
+      <c r="B6" s="18"/>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1223,10 +1235,10 @@
     <row r="15" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="17"/>
       <c r="B15" s="17"/>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="16" t="s">
         <v>196</v>
       </c>
     </row>
@@ -1404,17 +1416,17 @@
         <v>131</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A31" s="1">
+    <row r="31" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="15">
         <v>10</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D31" s="16" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1439,10 +1451,10 @@
       <c r="B33" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D33" s="19" t="s">
         <v>133</v>
       </c>
     </row>
@@ -1471,40 +1483,40 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="16">
+      <c r="A36" s="18">
         <v>14</v>
       </c>
-      <c r="B36" s="16" t="s">
+      <c r="B36" s="18" t="s">
         <v>52</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="16"/>
-      <c r="B37" s="16"/>
+      <c r="A37" s="18"/>
+      <c r="B37" s="18"/>
       <c r="C37" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D37" s="3"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="16"/>
-      <c r="B38" s="16"/>
+      <c r="A38" s="18"/>
+      <c r="B38" s="18"/>
       <c r="C38" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D38" s="3"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="16"/>
-      <c r="B39" s="16"/>
+      <c r="A39" s="18"/>
+      <c r="B39" s="18"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="16"/>
-      <c r="B40" s="16"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="18"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
     </row>
@@ -2054,6 +2066,36 @@
     </row>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A16:A22"/>
+    <mergeCell ref="B16:B22"/>
+    <mergeCell ref="A10:A15"/>
+    <mergeCell ref="B10:B15"/>
+    <mergeCell ref="B36:B40"/>
+    <mergeCell ref="A36:A40"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B47:B55"/>
+    <mergeCell ref="A47:A55"/>
+    <mergeCell ref="B56:B59"/>
+    <mergeCell ref="A56:A59"/>
+    <mergeCell ref="B41:B46"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="B60:B63"/>
+    <mergeCell ref="A60:A63"/>
+    <mergeCell ref="B64:B67"/>
+    <mergeCell ref="A64:A67"/>
+    <mergeCell ref="B68:B71"/>
+    <mergeCell ref="A68:A71"/>
     <mergeCell ref="B84:B86"/>
     <mergeCell ref="B87:B90"/>
     <mergeCell ref="A84:A86"/>
@@ -2064,36 +2106,6 @@
     <mergeCell ref="A76:A80"/>
     <mergeCell ref="A81:A83"/>
     <mergeCell ref="B81:B83"/>
-    <mergeCell ref="B60:B63"/>
-    <mergeCell ref="A60:A63"/>
-    <mergeCell ref="B64:B67"/>
-    <mergeCell ref="A64:A67"/>
-    <mergeCell ref="B68:B71"/>
-    <mergeCell ref="A68:A71"/>
-    <mergeCell ref="B47:B55"/>
-    <mergeCell ref="A47:A55"/>
-    <mergeCell ref="B56:B59"/>
-    <mergeCell ref="A56:A59"/>
-    <mergeCell ref="B41:B46"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="B36:B40"/>
-    <mergeCell ref="A36:A40"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A16:A22"/>
-    <mergeCell ref="B16:B22"/>
-    <mergeCell ref="A10:A15"/>
-    <mergeCell ref="B10:B15"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
EM-16.10 - Nova página para admistradores
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\EcommerceModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED3F14C-3E97-4F24-9C0B-06BB3B6D7915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5373D6B-09B7-430D-898D-9FA0F0EBE706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-900" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="200">
   <si>
     <t>US</t>
   </si>
@@ -619,6 +619,12 @@
   </si>
   <si>
     <t>Criar tela para o usuário visualizar individualmente os produtos</t>
+  </si>
+  <si>
+    <t>Criar tela para listar todas os menus de parametrizações do admin</t>
+  </si>
+  <si>
+    <t>16.10</t>
   </si>
 </sst>
 </file>
@@ -672,7 +678,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -720,6 +726,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1065,7 +1077,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
@@ -1088,10 +1100,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="18">
+      <c r="A2" s="20">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1100,8 +1112,8 @@
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="18"/>
-      <c r="B3" s="18"/>
+      <c r="A3" s="20"/>
+      <c r="B3" s="20"/>
       <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1110,8 +1122,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="18"/>
-      <c r="B4" s="18"/>
+      <c r="A4" s="20"/>
+      <c r="B4" s="20"/>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1120,8 +1132,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="18"/>
-      <c r="B5" s="18"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
       <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1130,8 +1142,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="18"/>
-      <c r="B6" s="18"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="20"/>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1140,10 +1152,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="17">
+      <c r="A7" s="19">
         <v>2</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="19" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -1154,8 +1166,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
+      <c r="A8" s="19"/>
+      <c r="B8" s="19"/>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1167,8 +1179,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="17"/>
-      <c r="B9" s="17"/>
+      <c r="A9" s="19"/>
+      <c r="B9" s="19"/>
       <c r="C9" s="6" t="s">
         <v>15</v>
       </c>
@@ -1178,10 +1190,10 @@
       <c r="E9" s="7"/>
     </row>
     <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17">
+      <c r="A10" s="19">
         <v>3</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="19" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1192,8 +1204,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="17"/>
-      <c r="B11" s="17"/>
+      <c r="A11" s="19"/>
+      <c r="B11" s="19"/>
       <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1202,8 +1214,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="17"/>
-      <c r="B12" s="17"/>
+      <c r="A12" s="19"/>
+      <c r="B12" s="19"/>
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
@@ -1212,8 +1224,8 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="17"/>
-      <c r="B13" s="17"/>
+      <c r="A13" s="19"/>
+      <c r="B13" s="19"/>
       <c r="C13" s="12" t="s">
         <v>21</v>
       </c>
@@ -1223,8 +1235,8 @@
       <c r="E13" s="11"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="17"/>
-      <c r="B14" s="17"/>
+      <c r="A14" s="19"/>
+      <c r="B14" s="19"/>
       <c r="C14" s="3" t="s">
         <v>23</v>
       </c>
@@ -1233,8 +1245,8 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17"/>
-      <c r="B15" s="17"/>
+      <c r="A15" s="19"/>
+      <c r="B15" s="19"/>
       <c r="C15" s="16" t="s">
         <v>197</v>
       </c>
@@ -1243,10 +1255,10 @@
       </c>
     </row>
     <row r="16" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17">
+      <c r="A16" s="19">
         <v>4</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="19" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="8" t="s">
@@ -1257,8 +1269,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17"/>
-      <c r="B17" s="17"/>
+      <c r="A17" s="19"/>
+      <c r="B17" s="19"/>
       <c r="C17" s="8" t="s">
         <v>191</v>
       </c>
@@ -1267,8 +1279,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17"/>
-      <c r="B18" s="17"/>
+      <c r="A18" s="19"/>
+      <c r="B18" s="19"/>
       <c r="C18" s="8" t="s">
         <v>194</v>
       </c>
@@ -1277,8 +1289,8 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="17"/>
-      <c r="B19" s="17"/>
+      <c r="A19" s="19"/>
+      <c r="B19" s="19"/>
       <c r="C19" s="9" t="s">
         <v>26</v>
       </c>
@@ -1287,8 +1299,8 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="17"/>
-      <c r="B20" s="17"/>
+      <c r="A20" s="19"/>
+      <c r="B20" s="19"/>
       <c r="C20" s="9" t="s">
         <v>28</v>
       </c>
@@ -1297,8 +1309,8 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="17"/>
-      <c r="B21" s="17"/>
+      <c r="A21" s="19"/>
+      <c r="B21" s="19"/>
       <c r="C21" s="10" t="s">
         <v>195</v>
       </c>
@@ -1307,8 +1319,8 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="17"/>
-      <c r="B22" s="17"/>
+      <c r="A22" s="19"/>
+      <c r="B22" s="19"/>
       <c r="C22" s="1" t="s">
         <v>29</v>
       </c>
@@ -1317,10 +1329,10 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="17">
+      <c r="A23" s="19">
         <v>5</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="19" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -1331,8 +1343,8 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="17"/>
-      <c r="B24" s="17"/>
+      <c r="A24" s="19"/>
+      <c r="B24" s="19"/>
       <c r="C24" s="1" t="s">
         <v>32</v>
       </c>
@@ -1341,10 +1353,10 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="17">
+      <c r="A25" s="19">
         <v>6</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="19" t="s">
         <v>33</v>
       </c>
       <c r="C25" s="1" t="s">
@@ -1355,8 +1367,8 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="17"/>
-      <c r="B26" s="17"/>
+      <c r="A26" s="19"/>
+      <c r="B26" s="19"/>
       <c r="C26" s="1" t="s">
         <v>35</v>
       </c>
@@ -1365,10 +1377,10 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="17">
+      <c r="A27" s="19">
         <v>7</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="19" t="s">
         <v>36</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -1379,8 +1391,8 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="17"/>
-      <c r="B28" s="17"/>
+      <c r="A28" s="19"/>
+      <c r="B28" s="19"/>
       <c r="C28" s="1" t="s">
         <v>38</v>
       </c>
@@ -1445,26 +1457,26 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="17">
+      <c r="A33" s="19">
         <v>12</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="C33" s="19" t="s">
+      <c r="C33" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="D33" s="19" t="s">
+      <c r="D33" s="17" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="34" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="17"/>
-      <c r="B34" s="17"/>
-      <c r="C34" s="2" t="s">
+      <c r="A34" s="19"/>
+      <c r="B34" s="19"/>
+      <c r="C34" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D34" s="17" t="s">
         <v>135</v>
       </c>
     </row>
@@ -1483,48 +1495,48 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="18">
+      <c r="A36" s="20">
         <v>14</v>
       </c>
-      <c r="B36" s="18" t="s">
+      <c r="B36" s="20" t="s">
         <v>52</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="18"/>
-      <c r="B37" s="18"/>
+      <c r="A37" s="20"/>
+      <c r="B37" s="20"/>
       <c r="C37" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D37" s="3"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="18"/>
-      <c r="B38" s="18"/>
+      <c r="A38" s="20"/>
+      <c r="B38" s="20"/>
       <c r="C38" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D38" s="3"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="18"/>
-      <c r="B39" s="18"/>
+      <c r="A39" s="20"/>
+      <c r="B39" s="20"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="18"/>
-      <c r="B40" s="18"/>
+      <c r="A40" s="20"/>
+      <c r="B40" s="20"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="17">
+      <c r="A41" s="19">
         <v>15</v>
       </c>
-      <c r="B41" s="17" t="s">
+      <c r="B41" s="19" t="s">
         <v>55</v>
       </c>
       <c r="C41" s="13" t="s">
@@ -1535,8 +1547,8 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="17"/>
-      <c r="B42" s="17"/>
+      <c r="A42" s="19"/>
+      <c r="B42" s="19"/>
       <c r="C42" s="13" t="s">
         <v>57</v>
       </c>
@@ -1545,8 +1557,8 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="17"/>
-      <c r="B43" s="17"/>
+      <c r="A43" s="19"/>
+      <c r="B43" s="19"/>
       <c r="C43" s="1" t="s">
         <v>58</v>
       </c>
@@ -1555,8 +1567,8 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="17"/>
-      <c r="B44" s="17"/>
+      <c r="A44" s="19"/>
+      <c r="B44" s="19"/>
       <c r="C44" s="13" t="s">
         <v>59</v>
       </c>
@@ -1565,8 +1577,8 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="17"/>
-      <c r="B45" s="17"/>
+      <c r="A45" s="19"/>
+      <c r="B45" s="19"/>
       <c r="C45" s="13" t="s">
         <v>60</v>
       </c>
@@ -1575,8 +1587,8 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="17"/>
-      <c r="B46" s="17"/>
+      <c r="A46" s="19"/>
+      <c r="B46" s="19"/>
       <c r="C46" s="1" t="s">
         <v>61</v>
       </c>
@@ -1584,483 +1596,493 @@
         <v>142</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="17">
+    <row r="47" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="19">
         <v>16</v>
       </c>
-      <c r="B47" s="17" t="s">
+      <c r="B47" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C47" s="21" t="s">
+        <v>198</v>
+      </c>
+      <c r="D47" s="21" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="19"/>
+      <c r="B48" s="19"/>
+      <c r="C48" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D47" s="1" t="s">
+      <c r="D48" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="17"/>
-      <c r="B48" s="17"/>
-      <c r="C48" s="1" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="19"/>
+      <c r="B49" s="19"/>
+      <c r="C49" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D48" s="1" t="s">
+      <c r="D49" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="17"/>
-      <c r="B49" s="17"/>
-      <c r="C49" s="1" t="s">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="19"/>
+      <c r="B50" s="19"/>
+      <c r="C50" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D49" s="2" t="s">
+      <c r="D50" s="2" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="17"/>
-      <c r="B50" s="17"/>
-      <c r="C50" s="1" t="s">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="19"/>
+      <c r="B51" s="19"/>
+      <c r="C51" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D50" s="2" t="s">
+      <c r="D51" s="2" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="17"/>
-      <c r="B51" s="17"/>
-      <c r="C51" s="1" t="s">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="19"/>
+      <c r="B52" s="19"/>
+      <c r="C52" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D51" s="2" t="s">
+      <c r="D52" s="2" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="17"/>
-      <c r="B52" s="17"/>
-      <c r="C52" s="1" t="s">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="19"/>
+      <c r="B53" s="19"/>
+      <c r="C53" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D52" s="2" t="s">
+      <c r="D53" s="2" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="17"/>
-      <c r="B53" s="17"/>
-      <c r="C53" s="1" t="s">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="19"/>
+      <c r="B54" s="19"/>
+      <c r="C54" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D53" s="2" t="s">
+      <c r="D54" s="2" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="17"/>
-      <c r="B54" s="17"/>
-      <c r="C54" s="1" t="s">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="19"/>
+      <c r="B55" s="19"/>
+      <c r="C55" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D54" s="2" t="s">
+      <c r="D55" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="17"/>
-      <c r="B55" s="17"/>
-      <c r="C55" s="1" t="s">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="19"/>
+      <c r="B56" s="19"/>
+      <c r="C56" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D55" s="2" t="s">
+      <c r="D56" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="17">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="19">
         <v>17</v>
       </c>
-      <c r="B56" s="17" t="s">
+      <c r="B57" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C57" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D56" s="1" t="s">
+      <c r="D57" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="17"/>
-      <c r="B57" s="17"/>
-      <c r="C57" s="1" t="s">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="19"/>
+      <c r="B58" s="19"/>
+      <c r="C58" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D57" s="1" t="s">
+      <c r="D58" s="1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="17"/>
-      <c r="B58" s="17"/>
-      <c r="C58" s="1" t="s">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="19"/>
+      <c r="B59" s="19"/>
+      <c r="C59" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D58" s="2" t="s">
+      <c r="D59" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="17"/>
-      <c r="B59" s="17"/>
-      <c r="C59" s="1" t="s">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="19"/>
+      <c r="B60" s="19"/>
+      <c r="C60" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D59" s="2" t="s">
+      <c r="D60" s="2" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="17">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="19">
         <v>18</v>
       </c>
-      <c r="B60" s="17" t="s">
+      <c r="B61" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="C60" s="1" t="s">
+      <c r="C61" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D60" s="1" t="s">
+      <c r="D61" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="17"/>
-      <c r="B61" s="17"/>
-      <c r="C61" s="1" t="s">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="19"/>
+      <c r="B62" s="19"/>
+      <c r="C62" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D61" s="1" t="s">
+      <c r="D62" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="17"/>
-      <c r="B62" s="17"/>
-      <c r="C62" s="1" t="s">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="19"/>
+      <c r="B63" s="19"/>
+      <c r="C63" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="D63" s="2" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="17"/>
-      <c r="B63" s="17"/>
-      <c r="C63" s="1" t="s">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="19"/>
+      <c r="B64" s="19"/>
+      <c r="C64" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D63" s="2" t="s">
+      <c r="D64" s="2" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A64" s="17">
+    <row r="65" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A65" s="19">
         <v>19</v>
       </c>
-      <c r="B64" s="17" t="s">
+      <c r="B65" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="C64" s="1" t="s">
+      <c r="C65" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D64" s="1" t="s">
+      <c r="D65" s="1" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="17"/>
-      <c r="B65" s="17"/>
-      <c r="C65" s="1" t="s">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="19"/>
+      <c r="B66" s="19"/>
+      <c r="C66" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D65" s="1" t="s">
+      <c r="D66" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="17"/>
-      <c r="B66" s="17"/>
-      <c r="C66" s="1" t="s">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="19"/>
+      <c r="B67" s="19"/>
+      <c r="C67" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D66" s="2" t="s">
+      <c r="D67" s="2" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="17"/>
-      <c r="B67" s="17"/>
-      <c r="C67" s="1" t="s">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="19"/>
+      <c r="B68" s="19"/>
+      <c r="C68" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D67" s="2" t="s">
+      <c r="D68" s="2" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="17">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="19">
         <v>20</v>
       </c>
-      <c r="B68" s="17" t="s">
+      <c r="B69" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="C68" s="1" t="s">
+      <c r="C69" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="D68" s="1" t="s">
+      <c r="D69" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="17"/>
-      <c r="B69" s="17"/>
-      <c r="C69" s="1" t="s">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="19"/>
+      <c r="B70" s="19"/>
+      <c r="C70" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D69" s="1" t="s">
+      <c r="D70" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="70" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A70" s="17"/>
-      <c r="B70" s="17"/>
-      <c r="C70" s="1" t="s">
+    <row r="71" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A71" s="19"/>
+      <c r="B71" s="19"/>
+      <c r="C71" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D70" s="2" t="s">
+      <c r="D71" s="2" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="17"/>
-      <c r="B71" s="17"/>
-      <c r="C71" s="1" t="s">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="19"/>
+      <c r="B72" s="19"/>
+      <c r="C72" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D71" s="2" t="s">
+      <c r="D72" s="2" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="17">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="19">
         <v>21</v>
       </c>
-      <c r="B72" s="17" t="s">
+      <c r="B73" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="C72" s="1" t="s">
+      <c r="C73" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D72" s="1" t="s">
+      <c r="D73" s="1" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="17"/>
-      <c r="B73" s="17"/>
-      <c r="C73" s="1" t="s">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="19"/>
+      <c r="B74" s="19"/>
+      <c r="C74" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D73" s="1" t="s">
+      <c r="D74" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="17"/>
-      <c r="B74" s="17"/>
-      <c r="C74" s="1" t="s">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="19"/>
+      <c r="B75" s="19"/>
+      <c r="C75" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D74" s="2" t="s">
+      <c r="D75" s="2" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="17"/>
-      <c r="B75" s="17"/>
-      <c r="C75" s="1" t="s">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="19"/>
+      <c r="B76" s="19"/>
+      <c r="C76" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D75" s="2" t="s">
+      <c r="D76" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="17">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="19">
         <v>22</v>
       </c>
-      <c r="B76" s="17" t="s">
+      <c r="B77" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="C76" s="1" t="s">
+      <c r="C77" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D76" s="1" t="s">
+      <c r="D77" s="1" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="17"/>
-      <c r="B77" s="17"/>
-      <c r="C77" s="1" t="s">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="19"/>
+      <c r="B78" s="19"/>
+      <c r="C78" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D77" s="1" t="s">
+      <c r="D78" s="1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="17"/>
-      <c r="B78" s="17"/>
-      <c r="C78" s="1" t="s">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="19"/>
+      <c r="B79" s="19"/>
+      <c r="C79" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D78" s="2" t="s">
+      <c r="D79" s="2" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="17"/>
-      <c r="B79" s="17"/>
-      <c r="C79" s="1" t="s">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="19"/>
+      <c r="B80" s="19"/>
+      <c r="C80" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D79" s="2" t="s">
+      <c r="D80" s="2" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="17"/>
-      <c r="B80" s="17"/>
-      <c r="C80" s="1" t="s">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="19"/>
+      <c r="B81" s="19"/>
+      <c r="C81" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D80" s="2" t="s">
+      <c r="D81" s="2" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="17">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" s="19">
         <v>23</v>
       </c>
-      <c r="B81" s="17" t="s">
+      <c r="B82" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="C81" s="1" t="s">
+      <c r="C82" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D81" s="1" t="s">
+      <c r="D82" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="17"/>
-      <c r="B82" s="17"/>
-      <c r="C82" s="1" t="s">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="19"/>
+      <c r="B83" s="19"/>
+      <c r="C83" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D82" s="1" t="s">
+      <c r="D83" s="1" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="17"/>
-      <c r="B83" s="17"/>
-      <c r="C83" s="1" t="s">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="19"/>
+      <c r="B84" s="19"/>
+      <c r="C84" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D83" s="1" t="s">
+      <c r="D84" s="1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="17">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="19">
         <v>24</v>
       </c>
-      <c r="B84" s="17" t="s">
+      <c r="B85" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C84" s="1" t="s">
+      <c r="C85" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D84" s="1" t="s">
+      <c r="D85" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="17"/>
-      <c r="B85" s="17"/>
-      <c r="C85" s="1" t="s">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="19"/>
+      <c r="B86" s="19"/>
+      <c r="C86" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D85" s="1" t="s">
+      <c r="D86" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="17"/>
-      <c r="B86" s="17"/>
-      <c r="C86" s="1" t="s">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="19"/>
+      <c r="B87" s="19"/>
+      <c r="C87" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D86" s="1" t="s">
+      <c r="D87" s="1" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="17">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="19">
         <v>25</v>
       </c>
-      <c r="B87" s="17" t="s">
+      <c r="B88" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="C87" s="1" t="s">
+      <c r="C88" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D87" s="1" t="s">
+      <c r="D88" s="1" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="17"/>
-      <c r="B88" s="17"/>
-      <c r="C88" s="1" t="s">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="19"/>
+      <c r="B89" s="19"/>
+      <c r="C89" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D88" s="1" t="s">
+      <c r="D89" s="1" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="17"/>
-      <c r="B89" s="17"/>
-      <c r="C89" s="1" t="s">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" s="19"/>
+      <c r="B90" s="19"/>
+      <c r="C90" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D89" s="1" t="s">
+      <c r="D90" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="17"/>
-      <c r="B90" s="17"/>
-      <c r="C90" s="1" t="s">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" s="19"/>
+      <c r="B91" s="19"/>
+      <c r="C91" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D90" s="1" t="s">
+      <c r="D91" s="1" t="s">
         <v>186</v>
       </c>
     </row>
@@ -2084,33 +2106,33 @@
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B47:B55"/>
-    <mergeCell ref="A47:A55"/>
-    <mergeCell ref="B56:B59"/>
-    <mergeCell ref="A56:A59"/>
+    <mergeCell ref="B57:B60"/>
+    <mergeCell ref="A57:A60"/>
     <mergeCell ref="B41:B46"/>
     <mergeCell ref="A41:A46"/>
-    <mergeCell ref="B60:B63"/>
-    <mergeCell ref="A60:A63"/>
-    <mergeCell ref="B64:B67"/>
-    <mergeCell ref="A64:A67"/>
-    <mergeCell ref="B68:B71"/>
-    <mergeCell ref="A68:A71"/>
-    <mergeCell ref="B84:B86"/>
-    <mergeCell ref="B87:B90"/>
-    <mergeCell ref="A84:A86"/>
-    <mergeCell ref="A87:A90"/>
-    <mergeCell ref="B72:B75"/>
-    <mergeCell ref="A72:A75"/>
-    <mergeCell ref="B76:B80"/>
-    <mergeCell ref="A76:A80"/>
-    <mergeCell ref="A81:A83"/>
-    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="B47:B56"/>
+    <mergeCell ref="A47:A56"/>
+    <mergeCell ref="B61:B64"/>
+    <mergeCell ref="A61:A64"/>
+    <mergeCell ref="B65:B68"/>
+    <mergeCell ref="A65:A68"/>
+    <mergeCell ref="B69:B72"/>
+    <mergeCell ref="A69:A72"/>
+    <mergeCell ref="B85:B87"/>
+    <mergeCell ref="B88:B91"/>
+    <mergeCell ref="A85:A87"/>
+    <mergeCell ref="A88:A91"/>
+    <mergeCell ref="B73:B76"/>
+    <mergeCell ref="A73:A76"/>
+    <mergeCell ref="B77:B81"/>
+    <mergeCell ref="A77:A81"/>
+    <mergeCell ref="A82:A84"/>
+    <mergeCell ref="B82:B84"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D2 C19:D19 B3:D6 C47 A56:C56 C48:C49 C53:C55 A60:C60 C58:C59 A64:C64 C62:C63 A68:C68 C66:C67 A72:C72 C70:C71 A76:C76 C74:C75 A81:C81 C78:C80 A84:C84 C83 A87:C87 C86 C90 A7:C7 A8:C8 A9:C9 A10:C10 C11 C12 C13 C14 A31:D31 C20 C22 A23:C23 A24:C24 A25:C25 A26:C26 A27:C27 A28:C28 A29:C29 A30:C30 A36:D40 A32:C32 A33:C33 A35:C35 A46:C46 A41:C41 A42:C42 A43:C43 A44:C44 A45:C45 C51 C52 C50 C57 C61 C65 C69 C73 C77 C82 C85 C88 C89" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D2 C19:D19 B3:D6 C48 A57:C57 C49:C50 C54:C56 A61:C61 C59:C60 A65:C65 C63:C64 A69:C69 C67:C68 A73:C73 C71:C72 A77:C77 C75:C76 A82:C82 C79:C81 A85:C85 C84 A88:C88 C87 C91 A7:C7 A8:C8 A9:C9 A10:C10 C11 C12 C13 C14 A31:D31 C20 C22 A23:C23 A24:C24 A25:C25 A26:C26 A27:C27 A28:C28 A29:C29 A30:C30 A36:D40 A32:C32 A33:C33 A35:C35 A46:C46 A41:C41 A42:C42 A43:C43 A44:C44 A45:C45 C52 C53 C51 C58 C62 C66 C70 C74 C78 C83 C86 C89 C90" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>